<commit_message>
Test: modify deal brief description to validate prod data flow
</commit_message>
<xml_diff>
--- a/public/data/d365_opps_export.xlsx
+++ b/public/data/d365_opps_export.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hans\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alithyaca-my.sharepoint.com/personal/hans_westphal_alithya_com/Documents/FY27/d365-personal-analytics-v2/public/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACDBC4EC-E1DB-4B7B-B85B-CE05B26A1773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{ACDBC4EC-E1DB-4B7B-B85B-CE05B26A1773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49DD3AB7-7BF9-49B2-A08F-3D8EA7A3638F}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -156,9 +156,6 @@
     <t>Northwind Digital</t>
   </si>
   <si>
-    <t>Contoso Technology Technologies, a Calgary-based leader in interactive collaboration solutions, is embarking on a transformative CRM migration project. The initiative, sponsored by Microsoft, involves transitioning from Salesforce, HubSpot, and CPQ systems to Dynamics 365 (D365) Sales and Customer Service, with the integration of Expert Logics ISV add-ons for advanced CPQ capabilities. The project is valued at $3.1M, with a targeted nine-month deployment and a go-live deadline in June. Avanade was initially quoted, but the CIO has requested Microsoft to identify an alternative partner, emphasizing the strategic importance of this migration. The budget is set at $1.5M, with $1.8M in ECIF funding available for two years, and annual licensing costs of $900K. Contoso Technology Technologies, a subsidiary of Foxconn, operates globally with a workforce of 600–1,000 employees and a mission to enable meaningful connections through AI-powered interactivity. The migration aims to unify sales, marketing, and support operations, streamline workflows, and enhance customer engagement. By leveraging D365’s advanced automation, analytics, and integration capabilities, Contoso Technology Technologies seeks to modernize its CRM landscape, drive operational efficiency, and support its growth in the education and enterprise sectors. This opportunity represents a pivotal step in Contoso Technology’s digital transformation journey, positioning the company to better serve its high-profile clients and maintain market leadership in interactive technology.</t>
-  </si>
-  <si>
     <t>Meeting Wednesday with Contoso Technology and MSFT to review proposal / Board meeting this week.</t>
   </si>
   <si>
@@ -1250,15 +1247,22 @@
   <si>
     <t>Probability</t>
   </si>
+  <si>
+    <t>PIPELINE TEST – SHOULD SHOW IN PROD</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1281,7 +1285,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1291,6 +1295,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1723,7 +1728,7 @@
         <v>13</v>
       </c>
       <c r="O1" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="P1" t="s">
         <v>14</v>
@@ -1871,11 +1876,11 @@
       <c r="E4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="H4" s="4">
         <v>46107.833333333343</v>
@@ -1887,7 +1892,7 @@
         <v>2391000</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M4" s="1" t="s">
         <v>26</v>
@@ -1906,30 +1911,30 @@
         <v>46103.74790509259</v>
       </c>
       <c r="S4" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:20" ht="29.15" customHeight="1">
       <c r="A5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>45</v>
       </c>
       <c r="C5" s="2">
         <v>46103.914872685193</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>49</v>
       </c>
       <c r="H5" s="4">
         <v>46121.833333333343</v>
@@ -1941,7 +1946,7 @@
         <v>96300</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="M5" s="1" t="s">
         <v>26</v>
@@ -1960,33 +1965,33 @@
         <v>46103.748206018521</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="S5" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:20" ht="409.6" customHeight="1">
       <c r="A6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>53</v>
       </c>
       <c r="C6" s="2">
         <v>46109.880787037036</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="H6" s="4">
         <v>46107.833333333343</v>
@@ -2014,30 +2019,30 @@
         <v>46109.714120370372</v>
       </c>
       <c r="S6" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:20" ht="409.6" customHeight="1">
       <c r="A7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>60</v>
       </c>
       <c r="C7" s="2">
         <v>46105.599699074082</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F7" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>63</v>
       </c>
       <c r="H7" s="4">
         <v>46107.833333333343</v>
@@ -2049,7 +2054,7 @@
         <v>129000</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="M7" s="1" t="s">
         <v>26</v>
@@ -2071,30 +2076,30 @@
         <v>28</v>
       </c>
       <c r="S7" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:20" ht="116.6" customHeight="1">
       <c r="A8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>66</v>
       </c>
       <c r="C8" s="2">
         <v>46109.750381944446</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="1" t="s">
         <v>69</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>70</v>
       </c>
       <c r="H8" s="4">
         <v>46107.833333333343</v>
@@ -2109,7 +2114,7 @@
         <v>26</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O8" s="6">
         <f t="shared" si="0"/>
@@ -2125,27 +2130,27 @@
         <v>28</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:20">
       <c r="A9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>73</v>
       </c>
       <c r="C9" s="2">
         <v>46109.621111111112</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>76</v>
       </c>
       <c r="H9" s="4">
         <v>46114.833333333343</v>
@@ -2160,7 +2165,7 @@
         <v>26</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O9" s="6">
         <f t="shared" si="0"/>
@@ -2173,30 +2178,30 @@
         <v>46109.454444444447</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:20" ht="43.75" customHeight="1">
       <c r="A10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="C10" s="2">
         <v>46104.021504629629</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F10" s="3" t="s">
+      <c r="G10" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>83</v>
       </c>
       <c r="H10" s="4">
         <v>46107.833333333343</v>
@@ -2211,7 +2216,7 @@
         <v>26</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O10" s="6">
         <f t="shared" si="0"/>
@@ -2224,30 +2229,30 @@
         <v>46103.854837962957</v>
       </c>
       <c r="S10" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="1:20" ht="116.6" customHeight="1">
       <c r="A11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>86</v>
       </c>
       <c r="C11" s="2">
         <v>46104.028715277767</v>
       </c>
       <c r="D11" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F11" s="3" t="s">
+      <c r="G11" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>89</v>
       </c>
       <c r="H11" s="4">
         <v>46107.833333333343</v>
@@ -2262,7 +2267,7 @@
         <v>26</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O11" s="6">
         <f t="shared" si="0"/>
@@ -2275,27 +2280,27 @@
         <v>46103.86204861111</v>
       </c>
       <c r="S11" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" spans="1:20">
       <c r="A12" t="s">
+        <v>90</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>92</v>
       </c>
       <c r="C12" s="2">
         <v>46091.595057870371</v>
       </c>
       <c r="D12" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>95</v>
       </c>
       <c r="H12" s="4">
         <v>46079.791666666657</v>
@@ -2307,13 +2312,13 @@
         <v>69800</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M12" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O12" s="6">
         <f t="shared" si="0"/>
@@ -2326,30 +2331,30 @@
         <v>46091.428391203714</v>
       </c>
       <c r="S12" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:20" ht="145.75" customHeight="1">
       <c r="A13" t="s">
+        <v>96</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>98</v>
       </c>
       <c r="C13" s="2">
         <v>46109.74454861111</v>
       </c>
       <c r="D13" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="G13" s="1" t="s">
         <v>101</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>102</v>
       </c>
       <c r="H13" s="4">
         <v>46107.833333333343</v>
@@ -2377,30 +2382,30 @@
         <v>46109.577881944453</v>
       </c>
       <c r="S13" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:20" ht="145.75" customHeight="1">
       <c r="A14" t="s">
+        <v>102</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>104</v>
       </c>
       <c r="C14" s="2">
         <v>46092.730868055558</v>
       </c>
       <c r="D14" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="F14" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="G14" s="1" t="s">
         <v>107</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>108</v>
       </c>
       <c r="H14" s="4">
         <v>46100.833333333343</v>
@@ -2415,7 +2420,7 @@
         <v>26</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O14" s="6">
         <f t="shared" si="0"/>
@@ -2428,30 +2433,30 @@
         <v>46092.564201388886</v>
       </c>
       <c r="S14" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:20" ht="116.6" customHeight="1">
       <c r="A15" t="s">
+        <v>108</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>109</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>110</v>
       </c>
       <c r="C15" s="2">
         <v>46109.622673611113</v>
       </c>
       <c r="D15" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="F15" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="G15" s="1" t="s">
         <v>113</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>114</v>
       </c>
       <c r="H15" s="4">
         <v>46107.833333333343</v>
@@ -2463,13 +2468,13 @@
         <v>871000</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M15" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O15" s="6">
         <f t="shared" si="0"/>
@@ -2485,30 +2490,30 @@
         <v>35</v>
       </c>
       <c r="S15" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16" spans="1:20" ht="364.3" customHeight="1">
       <c r="A16" t="s">
+        <v>115</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>117</v>
       </c>
       <c r="C16" s="2">
         <v>46085.81453703704</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="F16" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="G16" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>121</v>
       </c>
       <c r="H16" s="4">
         <v>46090.833333333343</v>
@@ -2523,7 +2528,7 @@
         <v>26</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O16" s="6">
         <f t="shared" si="0"/>
@@ -2536,30 +2541,30 @@
         <v>46085.606203703697</v>
       </c>
       <c r="S16" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" spans="1:19" ht="145.75" customHeight="1">
       <c r="A17" t="s">
+        <v>121</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>123</v>
       </c>
       <c r="C17" s="2">
         <v>46092.924409722233</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="G17" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>127</v>
       </c>
       <c r="H17" s="4">
         <v>46044.791666666657</v>
@@ -2574,7 +2579,7 @@
         <v>26</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O17" s="6">
         <f t="shared" si="0"/>
@@ -2587,30 +2592,30 @@
         <v>46092.757743055547</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="131.15" customHeight="1">
       <c r="A18" t="s">
+        <v>127</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>129</v>
       </c>
       <c r="C18" s="2">
         <v>46109.623738425929</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="F18" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="G18" s="1" t="s">
         <v>132</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>133</v>
       </c>
       <c r="H18" s="4">
         <v>46100.833333333343</v>
@@ -2625,7 +2630,7 @@
         <v>26</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O18" s="6">
         <f t="shared" si="0"/>
@@ -2638,30 +2643,30 @@
         <v>46109.457071759258</v>
       </c>
       <c r="S18" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:19" ht="102" customHeight="1">
       <c r="A19" t="s">
+        <v>133</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>134</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>135</v>
       </c>
       <c r="C19" s="2">
         <v>46084.939201388886</v>
       </c>
       <c r="D19" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="F19" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="G19" s="1" t="s">
         <v>138</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>139</v>
       </c>
       <c r="H19" s="4">
         <v>46079.791666666657</v>
@@ -2673,13 +2678,13 @@
         <v>42900</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="M19" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O19" s="6">
         <f t="shared" si="0"/>
@@ -2692,30 +2697,30 @@
         <v>46084.730868055558</v>
       </c>
       <c r="S19" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" spans="1:19" ht="145.75" customHeight="1">
       <c r="A20" t="s">
+        <v>140</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>142</v>
       </c>
       <c r="C20" s="2">
         <v>46084.652060185188</v>
       </c>
       <c r="D20" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="F20" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="G20" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>146</v>
       </c>
       <c r="H20" s="4">
         <v>46093.833333333343</v>
@@ -2730,7 +2735,7 @@
         <v>26</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O20" s="6">
         <f t="shared" si="0"/>
@@ -2743,30 +2748,30 @@
         <v>46084.443726851852</v>
       </c>
       <c r="S20" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="21" spans="1:19" ht="116.6" customHeight="1">
       <c r="A21" t="s">
+        <v>146</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>147</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>148</v>
       </c>
       <c r="C21" s="2">
         <v>46092.939074074071</v>
       </c>
       <c r="D21" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="F21" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="G21" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>152</v>
       </c>
       <c r="H21" s="4">
         <v>46093.833333333343</v>
@@ -2781,7 +2786,7 @@
         <v>26</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O21" s="6">
         <f t="shared" si="0"/>
@@ -2794,30 +2799,30 @@
         <v>46092.772407407407</v>
       </c>
       <c r="S21" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:19" ht="87.45" customHeight="1">
       <c r="A22" t="s">
+        <v>152</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>154</v>
       </c>
       <c r="C22" s="2">
         <v>46097.672395833331</v>
       </c>
       <c r="D22" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="E22" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="F22" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="G22" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>158</v>
       </c>
       <c r="H22" s="4">
         <v>46107.833333333343</v>
@@ -2832,7 +2837,7 @@
         <v>26</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O22" s="6">
         <f t="shared" si="0"/>
@@ -2845,30 +2850,30 @@
         <v>46097.505729166667</v>
       </c>
       <c r="S22" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" spans="1:19" ht="160.30000000000001" customHeight="1">
       <c r="A23" t="s">
+        <v>158</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>160</v>
       </c>
       <c r="C23" s="2">
         <v>46092.92459490741</v>
       </c>
       <c r="D23" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="F23" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="G23" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>164</v>
       </c>
       <c r="H23" s="4">
         <v>46100.833333333343</v>
@@ -2883,7 +2888,7 @@
         <v>26</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O23" s="6">
         <f t="shared" si="0"/>
@@ -2896,30 +2901,30 @@
         <v>46092.757928240739</v>
       </c>
       <c r="S23" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="24" spans="1:19" ht="145.75" customHeight="1">
       <c r="A24" t="s">
+        <v>164</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>166</v>
       </c>
       <c r="C24" s="2">
         <v>46092.904513888891</v>
       </c>
       <c r="D24" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="E24" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="F24" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="G24" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>170</v>
       </c>
       <c r="H24" s="4">
         <v>46142.833333333343</v>
@@ -2934,7 +2939,7 @@
         <v>26</v>
       </c>
       <c r="N24" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O24" s="6">
         <f t="shared" si="0"/>
@@ -2947,30 +2952,30 @@
         <v>46092.737847222219</v>
       </c>
       <c r="S24" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25" spans="1:19" ht="204" customHeight="1">
       <c r="A25" t="s">
+        <v>170</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>172</v>
       </c>
       <c r="C25" s="2">
         <v>46092.939305555563</v>
       </c>
       <c r="D25" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="F25" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="F25" s="3" t="s">
+      <c r="G25" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>176</v>
       </c>
       <c r="H25" s="4">
         <v>46114.833333333343</v>
@@ -2982,13 +2987,13 @@
         <v>54700</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M25" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O25" s="6">
         <f t="shared" si="0"/>
@@ -3001,33 +3006,33 @@
         <v>46092.772638888891</v>
       </c>
       <c r="R25" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="S25" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="1:19" ht="131.15" customHeight="1">
       <c r="A26" t="s">
+        <v>178</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>180</v>
       </c>
       <c r="C26" s="2">
         <v>46092.925995370373</v>
       </c>
       <c r="D26" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="E26" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="F26" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="F26" s="3" t="s">
+      <c r="G26" s="1" t="s">
         <v>183</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>184</v>
       </c>
       <c r="H26" s="4">
         <v>46107.833333333343</v>
@@ -3039,7 +3044,7 @@
         <v>293000</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="M26" s="1" t="s">
         <v>26</v>
@@ -3058,30 +3063,30 @@
         <v>46092.759328703702</v>
       </c>
       <c r="S26" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="27" spans="1:19" ht="409.6" customHeight="1">
       <c r="A27" t="s">
+        <v>185</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>186</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>187</v>
       </c>
       <c r="C27" s="2">
         <v>46103.988796296297</v>
       </c>
       <c r="D27" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F27" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="E27" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F27" s="3" t="s">
+      <c r="G27" s="1" t="s">
         <v>189</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>190</v>
       </c>
       <c r="H27" s="4">
         <v>46107.833333333343</v>
@@ -3096,7 +3101,7 @@
         <v>26</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O27" s="6">
         <f t="shared" si="0"/>
@@ -3109,30 +3114,30 @@
         <v>46103.822129629632</v>
       </c>
       <c r="S27" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:19" ht="29.15" customHeight="1">
       <c r="A28" t="s">
+        <v>190</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>191</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>192</v>
       </c>
       <c r="C28" s="2">
         <v>46092.937858796293</v>
       </c>
       <c r="D28" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="F28" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="E28" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="F28" s="3" t="s">
+      <c r="G28" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>195</v>
       </c>
       <c r="H28" s="4">
         <v>46037.791666666657</v>
@@ -3144,13 +3149,13 @@
         <v>62300</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="M28" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O28" s="6">
         <f t="shared" si="0"/>
@@ -3163,30 +3168,30 @@
         <v>46092.771192129629</v>
       </c>
       <c r="S28" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="29" spans="1:19" ht="409.6" customHeight="1">
       <c r="A29" t="s">
+        <v>196</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>197</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>198</v>
       </c>
       <c r="C29" s="2">
         <v>46109.60869212963</v>
       </c>
       <c r="D29" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="F29" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="F29" s="3" t="s">
+      <c r="G29" s="1" t="s">
         <v>201</v>
-      </c>
-      <c r="G29" s="1" t="s">
-        <v>202</v>
       </c>
       <c r="H29" s="4">
         <v>46135.833333333343</v>
@@ -3201,7 +3206,7 @@
         <v>26</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O29" s="6">
         <f t="shared" si="0"/>
@@ -3214,30 +3219,30 @@
         <v>46109.442025462973</v>
       </c>
       <c r="S29" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="30" spans="1:19" ht="116.6" customHeight="1">
       <c r="A30" t="s">
+        <v>202</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>203</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>204</v>
       </c>
       <c r="C30" s="2">
         <v>46109.610173611109</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F30" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="G30" s="1" t="s">
         <v>206</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>207</v>
       </c>
       <c r="H30" s="4">
         <v>46107.833333333343</v>
@@ -3252,7 +3257,7 @@
         <v>26</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O30" s="6">
         <f t="shared" si="0"/>
@@ -3265,27 +3270,27 @@
         <v>46109.443506944437</v>
       </c>
       <c r="S30" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="31" spans="1:19">
       <c r="A31" t="s">
+        <v>207</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>208</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>209</v>
       </c>
       <c r="C31" s="2">
         <v>46109.610590277778</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>39</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H31" s="4">
         <v>46107.833333333343</v>
@@ -3297,13 +3302,13 @@
         <v>113000</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M31" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O31" s="6">
         <f t="shared" si="0"/>
@@ -3316,24 +3321,24 @@
         <v>46109.443923611107</v>
       </c>
       <c r="S31" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="32" spans="1:19">
       <c r="A32" t="s">
+        <v>211</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>213</v>
       </c>
       <c r="C32" s="2">
         <v>46109.618576388893</v>
       </c>
       <c r="D32" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="E32" s="1" t="s">
         <v>214</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>215</v>
       </c>
       <c r="H32" s="4">
         <v>46058.791666666657</v>
@@ -3348,7 +3353,7 @@
         <v>26</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O32" s="6">
         <f t="shared" si="0"/>
@@ -3361,30 +3366,30 @@
         <v>46109.451909722222</v>
       </c>
       <c r="S32" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="33" spans="1:19" ht="102" customHeight="1">
       <c r="A33" t="s">
+        <v>215</v>
+      </c>
+      <c r="B33" s="1" t="s">
         <v>216</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>217</v>
       </c>
       <c r="C33" s="2">
         <v>46109.610821759263</v>
       </c>
       <c r="D33" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E33" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="F33" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="G33" s="1" t="s">
         <v>220</v>
-      </c>
-      <c r="G33" s="1" t="s">
-        <v>221</v>
       </c>
       <c r="H33" s="4">
         <v>45890.833333333343</v>
@@ -3396,13 +3401,13 @@
         <v>48200</v>
       </c>
       <c r="L33" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="M33" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O33" s="6">
         <f t="shared" si="0"/>
@@ -3415,30 +3420,30 @@
         <v>46109.444155092591</v>
       </c>
       <c r="S33" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="34" spans="1:19" ht="409.6" customHeight="1">
       <c r="A34" t="s">
+        <v>222</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>223</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>224</v>
       </c>
       <c r="C34" s="2">
         <v>46109.611643518518</v>
       </c>
       <c r="D34" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="E34" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="F34" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="F34" s="3" t="s">
+      <c r="G34" s="1" t="s">
         <v>227</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>228</v>
       </c>
       <c r="H34" s="4">
         <v>46093.833333333343</v>
@@ -3450,13 +3455,13 @@
         <v>64300</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="M34" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O34" s="6">
         <f t="shared" ref="O34:O61" si="1">IF(S34="","",VALUE(LEFT(S34,FIND("%",S34)-1)))</f>
@@ -3469,30 +3474,30 @@
         <v>46109.444976851853</v>
       </c>
       <c r="S34" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="35" spans="1:19" ht="116.6" customHeight="1">
       <c r="A35" t="s">
+        <v>229</v>
+      </c>
+      <c r="B35" s="1" t="s">
         <v>230</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>231</v>
       </c>
       <c r="C35" s="2">
         <v>46109.619120370371</v>
       </c>
       <c r="D35" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="E35" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="F35" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="F35" s="3" t="s">
+      <c r="G35" s="1" t="s">
         <v>234</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>235</v>
       </c>
       <c r="H35" s="4">
         <v>46138.833333333343</v>
@@ -3507,7 +3512,7 @@
         <v>26</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O35" s="6">
         <f t="shared" si="1"/>
@@ -3520,30 +3525,30 @@
         <v>46109.452453703707</v>
       </c>
       <c r="S35" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="36" spans="1:19" ht="43.75" customHeight="1">
       <c r="A36" t="s">
+        <v>235</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>236</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>237</v>
       </c>
       <c r="C36" s="2">
         <v>46109.619351851848</v>
       </c>
       <c r="D36" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="E36" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="F36" s="3" t="s">
         <v>239</v>
       </c>
-      <c r="F36" s="3" t="s">
+      <c r="G36" s="1" t="s">
         <v>240</v>
-      </c>
-      <c r="G36" s="1" t="s">
-        <v>241</v>
       </c>
       <c r="H36" s="4">
         <v>46261.833333333343</v>
@@ -3558,7 +3563,7 @@
         <v>26</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O36" s="6">
         <f t="shared" si="1"/>
@@ -3571,27 +3576,27 @@
         <v>46109.452685185177</v>
       </c>
       <c r="R36" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="S36" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="37" spans="1:19">
       <c r="A37" t="s">
+        <v>241</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>242</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>243</v>
       </c>
       <c r="C37" s="2">
         <v>46109.613946759258</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I37" s="4">
         <v>46293</v>
@@ -3603,7 +3608,7 @@
         <v>26</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O37" s="6">
         <f t="shared" si="1"/>
@@ -3616,30 +3621,30 @@
         <v>46109.447280092587</v>
       </c>
       <c r="S37" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="38" spans="1:19" ht="29.15" customHeight="1">
       <c r="A38" t="s">
+        <v>244</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>245</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>246</v>
       </c>
       <c r="C38" s="2">
         <v>46109.614317129628</v>
       </c>
       <c r="D38" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="E38" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="F38" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="F38" s="3" t="s">
+      <c r="G38" s="1" t="s">
         <v>249</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>250</v>
       </c>
       <c r="H38" s="4">
         <v>46021.791666666657</v>
@@ -3654,7 +3659,7 @@
         <v>26</v>
       </c>
       <c r="N38" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O38" s="6">
         <f t="shared" si="1"/>
@@ -3667,30 +3672,30 @@
         <v>46109.447650462957</v>
       </c>
       <c r="S38" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="39" spans="1:19" ht="247.75" customHeight="1">
       <c r="A39" t="s">
+        <v>250</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>251</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>252</v>
       </c>
       <c r="C39" s="2">
         <v>46109.614664351851</v>
       </c>
       <c r="D39" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="E39" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="F39" s="3" t="s">
         <v>254</v>
       </c>
-      <c r="F39" s="3" t="s">
+      <c r="G39" s="1" t="s">
         <v>255</v>
-      </c>
-      <c r="G39" s="1" t="s">
-        <v>256</v>
       </c>
       <c r="H39" s="4">
         <v>46051.791666666657</v>
@@ -3705,7 +3710,7 @@
         <v>26</v>
       </c>
       <c r="N39" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O39" s="6">
         <f t="shared" si="1"/>
@@ -3718,30 +3723,30 @@
         <v>46109.447997685187</v>
       </c>
       <c r="S39" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="40" spans="1:19">
       <c r="A40" t="s">
+        <v>256</v>
+      </c>
+      <c r="B40" s="1" t="s">
         <v>257</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>258</v>
       </c>
       <c r="C40" s="2">
         <v>46109.614907407413</v>
       </c>
       <c r="D40" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="E40" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="E40" s="1" t="s">
+      <c r="F40" s="3" t="s">
         <v>260</v>
       </c>
-      <c r="F40" s="3" t="s">
+      <c r="G40" s="1" t="s">
         <v>261</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>262</v>
       </c>
       <c r="H40" s="4">
         <v>46114.833333333343</v>
@@ -3753,13 +3758,13 @@
         <v>34300</v>
       </c>
       <c r="L40" s="1" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="M40" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N40" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O40" s="6">
         <f t="shared" si="1"/>
@@ -3772,30 +3777,30 @@
         <v>46109.448240740741</v>
       </c>
       <c r="S40" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="41" spans="1:19" ht="131.15" customHeight="1">
       <c r="A41" t="s">
+        <v>263</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>264</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>265</v>
       </c>
       <c r="C41" s="2">
         <v>46109.615717592591</v>
       </c>
       <c r="D41" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E41" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="F41" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="F41" s="3" t="s">
+      <c r="G41" s="1" t="s">
         <v>268</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>269</v>
       </c>
       <c r="H41" s="4">
         <v>46044.791666666657</v>
@@ -3810,7 +3815,7 @@
         <v>26</v>
       </c>
       <c r="N41" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O41" s="6">
         <f t="shared" si="1"/>
@@ -3823,30 +3828,30 @@
         <v>46109.449050925927</v>
       </c>
       <c r="S41" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="42" spans="1:19" ht="58.3" customHeight="1">
       <c r="A42" t="s">
+        <v>269</v>
+      </c>
+      <c r="B42" s="1" t="s">
         <v>270</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>271</v>
       </c>
       <c r="C42" s="2">
         <v>46109.616018518522</v>
       </c>
       <c r="D42" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F42" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="E42" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="F42" s="3" t="s">
+      <c r="G42" s="1" t="s">
         <v>273</v>
-      </c>
-      <c r="G42" s="1" t="s">
-        <v>274</v>
       </c>
       <c r="H42" s="4">
         <v>46166.833333333343</v>
@@ -3858,13 +3863,13 @@
         <v>192000</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M42" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O42" s="6">
         <f t="shared" si="1"/>
@@ -3877,30 +3882,30 @@
         <v>46109.44935185185</v>
       </c>
       <c r="S42" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="43" spans="1:19">
       <c r="A43" t="s">
+        <v>274</v>
+      </c>
+      <c r="B43" s="1" t="s">
         <v>275</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>276</v>
       </c>
       <c r="C43" s="2">
         <v>46109.61886574074</v>
       </c>
       <c r="D43" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="E43" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="F43" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="F43" s="3" t="s">
+      <c r="G43" s="1" t="s">
         <v>279</v>
-      </c>
-      <c r="G43" s="1" t="s">
-        <v>280</v>
       </c>
       <c r="H43" s="4">
         <v>46163.833333333343</v>
@@ -3912,13 +3917,13 @@
         <v>86400</v>
       </c>
       <c r="L43" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="M43" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N43" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O43" s="6">
         <f t="shared" si="1"/>
@@ -3931,30 +3936,30 @@
         <v>46109.452199074083</v>
       </c>
       <c r="S43" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="44" spans="1:19" ht="29.15" customHeight="1">
       <c r="A44" t="s">
+        <v>281</v>
+      </c>
+      <c r="B44" s="1" t="s">
         <v>282</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>283</v>
       </c>
       <c r="C44" s="2">
         <v>46109.616550925923</v>
       </c>
       <c r="D44" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E44" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="E44" s="1" t="s">
+      <c r="F44" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="F44" s="3" t="s">
+      <c r="G44" s="1" t="s">
         <v>286</v>
-      </c>
-      <c r="G44" s="1" t="s">
-        <v>287</v>
       </c>
       <c r="H44" s="4">
         <v>46100.833333333343</v>
@@ -3966,13 +3971,13 @@
         <v>150000</v>
       </c>
       <c r="L44" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="M44" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N44" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O44" s="6">
         <f t="shared" si="1"/>
@@ -3985,30 +3990,30 @@
         <v>46109.449884259258</v>
       </c>
       <c r="S44" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="45" spans="1:19" ht="87.45" customHeight="1">
       <c r="A45" t="s">
+        <v>288</v>
+      </c>
+      <c r="B45" s="1" t="s">
         <v>289</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>290</v>
       </c>
       <c r="C45" s="2">
         <v>46109.616851851853</v>
       </c>
       <c r="D45" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F45" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="E45" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="F45" s="3" t="s">
+      <c r="G45" s="1" t="s">
         <v>292</v>
-      </c>
-      <c r="G45" s="1" t="s">
-        <v>293</v>
       </c>
       <c r="H45" s="4">
         <v>46079.791666666657</v>
@@ -4020,13 +4025,13 @@
         <v>144000</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="M45" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N45" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O45" s="6">
         <f t="shared" si="1"/>
@@ -4039,30 +4044,30 @@
         <v>46109.450185185182</v>
       </c>
       <c r="S45" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="46" spans="1:19" ht="102" customHeight="1">
       <c r="A46" t="s">
+        <v>294</v>
+      </c>
+      <c r="B46" s="1" t="s">
         <v>295</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>296</v>
       </c>
       <c r="C46" s="2">
         <v>46109.617152777777</v>
       </c>
       <c r="D46" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="E46" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="F46" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="F46" s="3" t="s">
+      <c r="G46" s="1" t="s">
         <v>299</v>
-      </c>
-      <c r="G46" s="1" t="s">
-        <v>300</v>
       </c>
       <c r="H46" s="4">
         <v>46080.791666666657</v>
@@ -4074,13 +4079,13 @@
         <v>174000</v>
       </c>
       <c r="L46" s="1" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="M46" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N46" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O46" s="6">
         <f t="shared" si="1"/>
@@ -4093,30 +4098,30 @@
         <v>46109.450486111113</v>
       </c>
       <c r="S46" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="47" spans="1:19" ht="87.45" customHeight="1">
       <c r="A47" t="s">
+        <v>301</v>
+      </c>
+      <c r="B47" s="1" t="s">
         <v>302</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>303</v>
       </c>
       <c r="C47" s="2">
         <v>46109.617430555547</v>
       </c>
       <c r="D47" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F47" s="3" t="s">
         <v>304</v>
       </c>
-      <c r="E47" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="F47" s="3" t="s">
-        <v>305</v>
-      </c>
       <c r="G47" s="1" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="H47" s="4">
         <v>46079.791666666657</v>
@@ -4128,13 +4133,13 @@
         <v>20000</v>
       </c>
       <c r="L47" s="1" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="M47" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N47" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O47" s="6">
         <f t="shared" si="1"/>
@@ -4147,30 +4152,30 @@
         <v>46109.45076388889</v>
       </c>
       <c r="S47" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="48" spans="1:19" ht="43.75" customHeight="1">
       <c r="A48" t="s">
+        <v>305</v>
+      </c>
+      <c r="B48" s="1" t="s">
         <v>306</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>307</v>
       </c>
       <c r="C48" s="2">
         <v>46109.617650462962</v>
       </c>
       <c r="D48" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F48" s="3" t="s">
         <v>308</v>
       </c>
-      <c r="E48" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="F48" s="3" t="s">
+      <c r="G48" s="1" t="s">
         <v>309</v>
-      </c>
-      <c r="G48" s="1" t="s">
-        <v>310</v>
       </c>
       <c r="H48" s="4">
         <v>46079.791666666657</v>
@@ -4182,13 +4187,13 @@
         <v>57000</v>
       </c>
       <c r="L48" s="1" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="M48" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N48" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O48" s="6">
         <f t="shared" si="1"/>
@@ -4201,30 +4206,30 @@
         <v>46109.450983796298</v>
       </c>
       <c r="S48" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="49" spans="1:19" ht="29.15" customHeight="1">
       <c r="A49" t="s">
+        <v>310</v>
+      </c>
+      <c r="B49" s="1" t="s">
         <v>311</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>312</v>
       </c>
       <c r="C49" s="2">
         <v>46109.618298611109</v>
       </c>
       <c r="D49" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="E49" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="F49" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="F49" s="3" t="s">
+      <c r="G49" s="1" t="s">
         <v>315</v>
-      </c>
-      <c r="G49" s="1" t="s">
-        <v>316</v>
       </c>
       <c r="H49" s="4">
         <v>46093.833333333343</v>
@@ -4236,13 +4241,13 @@
         <v>46300</v>
       </c>
       <c r="L49" s="1" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="M49" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N49" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O49" s="6">
         <f t="shared" si="1"/>
@@ -4255,30 +4260,30 @@
         <v>46109.451631944437</v>
       </c>
       <c r="S49" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="50" spans="1:19" ht="43.75" customHeight="1">
       <c r="A50" t="s">
+        <v>317</v>
+      </c>
+      <c r="B50" s="1" t="s">
         <v>318</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>319</v>
       </c>
       <c r="C50" s="2">
         <v>46092.908356481479</v>
       </c>
       <c r="D50" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="F50" s="3" t="s">
         <v>320</v>
       </c>
-      <c r="E50" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="F50" s="3" t="s">
+      <c r="G50" s="1" t="s">
         <v>321</v>
-      </c>
-      <c r="G50" s="1" t="s">
-        <v>322</v>
       </c>
       <c r="H50" s="4">
         <v>46271.833333333343</v>
@@ -4290,13 +4295,13 @@
         <v>0</v>
       </c>
       <c r="L50" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="M50" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N50" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O50" s="6">
         <f t="shared" si="1"/>
@@ -4309,30 +4314,30 @@
         <v>46092.741689814808</v>
       </c>
       <c r="S50" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="51" spans="1:19" ht="29.15" customHeight="1">
       <c r="A51" t="s">
+        <v>322</v>
+      </c>
+      <c r="B51" s="1" t="s">
         <v>323</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>324</v>
       </c>
       <c r="C51" s="2">
         <v>46108.883298611108</v>
       </c>
       <c r="D51" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="E51" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="E51" s="1" t="s">
+      <c r="F51" s="3" t="s">
         <v>326</v>
       </c>
-      <c r="F51" s="3" t="s">
+      <c r="G51" s="1" t="s">
         <v>327</v>
-      </c>
-      <c r="G51" s="1" t="s">
-        <v>328</v>
       </c>
       <c r="H51" s="4">
         <v>46121.833333333343</v>
@@ -4347,7 +4352,7 @@
         <v>26</v>
       </c>
       <c r="N51" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O51" s="6">
         <f t="shared" si="1"/>
@@ -4360,30 +4365,30 @@
         <v>46108.716631944437</v>
       </c>
       <c r="S51" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="52" spans="1:19" ht="43.75" customHeight="1">
       <c r="A52" t="s">
+        <v>328</v>
+      </c>
+      <c r="B52" s="1" t="s">
         <v>329</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>330</v>
       </c>
       <c r="C52" s="2">
         <v>46109.623437499999</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F52" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="G52" s="1" t="s">
         <v>332</v>
-      </c>
-      <c r="G52" s="1" t="s">
-        <v>333</v>
       </c>
       <c r="H52" s="4">
         <v>46072.791666666657</v>
@@ -4401,7 +4406,7 @@
         <v>26</v>
       </c>
       <c r="N52" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O52" s="6">
         <f t="shared" si="1"/>
@@ -4414,30 +4419,30 @@
         <v>46109.456770833327</v>
       </c>
       <c r="S52" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="53" spans="1:19" ht="160.30000000000001" customHeight="1">
       <c r="A53" t="s">
+        <v>333</v>
+      </c>
+      <c r="B53" s="1" t="s">
         <v>334</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>335</v>
       </c>
       <c r="C53" s="2">
         <v>46109.620324074072</v>
       </c>
       <c r="D53" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="E53" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="E53" s="1" t="s">
+      <c r="F53" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="F53" s="3" t="s">
+      <c r="G53" s="1" t="s">
         <v>338</v>
-      </c>
-      <c r="G53" s="1" t="s">
-        <v>339</v>
       </c>
       <c r="H53" s="4">
         <v>46149.833333333343</v>
@@ -4449,13 +4454,13 @@
         <v>45200</v>
       </c>
       <c r="L53" s="1" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="M53" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N53" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O53" s="6">
         <f t="shared" si="1"/>
@@ -4468,30 +4473,30 @@
         <v>46109.453657407408</v>
       </c>
       <c r="S53" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="54" spans="1:19" ht="43.75" customHeight="1">
       <c r="A54" t="s">
+        <v>340</v>
+      </c>
+      <c r="B54" s="1" t="s">
         <v>341</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>342</v>
       </c>
       <c r="C54" s="2">
         <v>46109.620671296303</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F54" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="G54" s="1" t="s">
         <v>344</v>
-      </c>
-      <c r="G54" s="1" t="s">
-        <v>345</v>
       </c>
       <c r="H54" s="4">
         <v>46208.833333333343</v>
@@ -4503,13 +4508,13 @@
         <v>222000</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="M54" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N54" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O54" s="6">
         <f t="shared" si="1"/>
@@ -4522,27 +4527,27 @@
         <v>46109.454004629632</v>
       </c>
       <c r="S54" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="55" spans="1:19">
       <c r="A55" t="s">
+        <v>345</v>
+      </c>
+      <c r="B55" s="1" t="s">
         <v>346</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>347</v>
       </c>
       <c r="C55" s="2">
         <v>46109.630381944437</v>
       </c>
       <c r="D55" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="E55" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="E55" s="1" t="s">
+      <c r="G55" s="1" t="s">
         <v>349</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>350</v>
       </c>
       <c r="H55" s="4">
         <v>46121.833333333343</v>
@@ -4557,7 +4562,7 @@
         <v>26</v>
       </c>
       <c r="N55" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O55" s="6">
         <f t="shared" si="1"/>
@@ -4570,27 +4575,27 @@
         <v>46109.46371527778</v>
       </c>
       <c r="S55" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="56" spans="1:19">
       <c r="A56" t="s">
+        <v>350</v>
+      </c>
+      <c r="B56" s="1" t="s">
         <v>351</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>352</v>
       </c>
       <c r="C56" s="2">
         <v>46109.612812500003</v>
       </c>
       <c r="D56" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="E56" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E56" s="1" t="s">
+      <c r="G56" s="1" t="s">
         <v>354</v>
-      </c>
-      <c r="G56" s="1" t="s">
-        <v>355</v>
       </c>
       <c r="H56" s="4">
         <v>46051.791666666657</v>
@@ -4602,13 +4607,13 @@
         <v>0</v>
       </c>
       <c r="L56" s="1" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M56" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N56" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O56" s="6">
         <f t="shared" si="1"/>
@@ -4621,30 +4626,30 @@
         <v>46109.446145833332</v>
       </c>
       <c r="S56" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="57" spans="1:19">
       <c r="A57" t="s">
+        <v>356</v>
+      </c>
+      <c r="B57" s="1" t="s">
         <v>357</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>358</v>
       </c>
       <c r="C57" s="2">
         <v>46109.613194444442</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>39</v>
       </c>
       <c r="F57" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="G57" s="1" t="s">
         <v>360</v>
-      </c>
-      <c r="G57" s="1" t="s">
-        <v>361</v>
       </c>
       <c r="H57" s="4">
         <v>46107.833333333343</v>
@@ -4656,13 +4661,13 @@
         <v>288000</v>
       </c>
       <c r="L57" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M57" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N57" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O57" s="6">
         <f t="shared" si="1"/>
@@ -4675,30 +4680,30 @@
         <v>46109.446527777778</v>
       </c>
       <c r="S57" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="58" spans="1:19" ht="87.45" customHeight="1">
       <c r="A58" t="s">
+        <v>361</v>
+      </c>
+      <c r="B58" s="1" t="s">
         <v>362</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>363</v>
       </c>
       <c r="C58" s="2">
         <v>46092.938900462963</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F58" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="G58" s="1" t="s">
         <v>365</v>
-      </c>
-      <c r="G58" s="1" t="s">
-        <v>366</v>
       </c>
       <c r="H58" s="4">
         <v>46100.833333333343</v>
@@ -4710,13 +4715,13 @@
         <v>85200</v>
       </c>
       <c r="L58" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="M58" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N58" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O58" s="6">
         <f t="shared" si="1"/>
@@ -4729,30 +4734,30 @@
         <v>46092.772233796299</v>
       </c>
       <c r="S58" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="59" spans="1:19" ht="189.45" customHeight="1">
       <c r="A59" t="s">
+        <v>366</v>
+      </c>
+      <c r="B59" s="1" t="s">
         <v>367</v>
-      </c>
-      <c r="B59" s="1" t="s">
-        <v>368</v>
       </c>
       <c r="C59" s="2">
         <v>46109.615416666667</v>
       </c>
       <c r="D59" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="E59" s="1" t="s">
         <v>369</v>
       </c>
-      <c r="E59" s="1" t="s">
+      <c r="F59" s="3" t="s">
         <v>370</v>
       </c>
-      <c r="F59" s="3" t="s">
+      <c r="G59" s="1" t="s">
         <v>371</v>
-      </c>
-      <c r="G59" s="1" t="s">
-        <v>372</v>
       </c>
       <c r="H59" s="4">
         <v>46100.833333333343</v>
@@ -4764,13 +4769,13 @@
         <v>53900</v>
       </c>
       <c r="L59" s="1" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="M59" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N59" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O59" s="6">
         <f t="shared" si="1"/>
@@ -4783,30 +4788,30 @@
         <v>46109.448750000003</v>
       </c>
       <c r="S59" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="60" spans="1:19" ht="306" customHeight="1">
       <c r="A60" t="s">
+        <v>373</v>
+      </c>
+      <c r="B60" s="1" t="s">
         <v>374</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>375</v>
       </c>
       <c r="C60" s="2">
         <v>46092.557858796303</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>39</v>
       </c>
       <c r="F60" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="G60" s="1" t="s">
         <v>377</v>
-      </c>
-      <c r="G60" s="1" t="s">
-        <v>378</v>
       </c>
       <c r="H60" s="4">
         <v>46425.791666666657</v>
@@ -4818,13 +4823,13 @@
         <v>65400</v>
       </c>
       <c r="L60" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M60" s="1" t="s">
         <v>26</v>
       </c>
       <c r="N60" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O60" s="6">
         <f t="shared" si="1"/>
@@ -4837,27 +4842,27 @@
         <v>46092.391192129631</v>
       </c>
       <c r="S60" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="61" spans="1:19">
       <c r="A61" t="s">
+        <v>378</v>
+      </c>
+      <c r="B61" s="1" t="s">
         <v>379</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>380</v>
       </c>
       <c r="C61" s="2">
         <v>46109.611284722218</v>
       </c>
       <c r="D61" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="E61" s="1" t="s">
         <v>381</v>
       </c>
-      <c r="E61" s="1" t="s">
+      <c r="G61" s="1" t="s">
         <v>382</v>
-      </c>
-      <c r="G61" s="1" t="s">
-        <v>383</v>
       </c>
       <c r="H61" s="4">
         <v>46100.833333333343</v>
@@ -4872,7 +4877,7 @@
         <v>26</v>
       </c>
       <c r="N61" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O61" s="6">
         <f t="shared" si="1"/>
@@ -4885,7 +4890,7 @@
         <v>46109.444618055553</v>
       </c>
       <c r="S61" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -4897,7 +4902,7 @@
       <formula1>300</formula1>
     </dataValidation>
     <dataValidation showInputMessage="1" showErrorMessage="1" error=" " promptTitle="Lookup (required)" prompt="This Account record must already exist in Microsoft Dynamics 365 or in this source file." sqref="E2:E1048576" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
-    <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Length Exceeded" error="This value must be less than or equal to 2000 characters long." promptTitle="Text" prompt="Maximum Length: 2000 characters." sqref="F2:F1048576" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Length Exceeded" error="This value must be less than or equal to 2000 characters long." promptTitle="Text" prompt="Maximum Length: 2000 characters." sqref="F2:F3 F5:F1048576" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>2000</formula1>
     </dataValidation>
     <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Length Exceeded" error="This value must be less than or equal to 10000 characters long." promptTitle="Text" prompt="Maximum Length: 10000 characters." sqref="G2:G1048576" xr:uid="{00000000-0002-0000-0000-000004000000}">
@@ -4941,46 +4946,46 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
+        <v>384</v>
+      </c>
+      <c r="B2" t="s">
         <v>385</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>386</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>387</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>388</v>
-      </c>
-      <c r="E2" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
+        <v>389</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" t="s">
         <v>390</v>
-      </c>
-      <c r="B3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D4" t="s">
         <v>27</v>
@@ -4988,16 +4993,16 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E5" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
Updated opportunity details to be less verbose and max 333 characters is length
</commit_message>
<xml_diff>
--- a/public/data/d365_opps_export.xlsx
+++ b/public/data/d365_opps_export.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alithyaca-my.sharepoint.com/personal/hans_westphal_alithya_com/Documents/FY27/d365-personal-analytics-v2/public/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{ACDBC4EC-E1DB-4B7B-B85B-CE05B26A1773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49DD3AB7-7BF9-49B2-A08F-3D8EA7A3638F}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{ACDBC4EC-E1DB-4B7B-B85B-CE05B26A1773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1FF97411-215C-4607-9230-AD8BAA0C9289}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="394">
   <si>
     <t>(Do Not Modify) Opportunity</t>
   </si>
@@ -105,9 +105,6 @@
     <t>Contoso Financial</t>
   </si>
   <si>
-    <t>D365 CE 8.2 to 9.1 Onprem migration</t>
-  </si>
-  <si>
     <t>Waiting on SOW signature sync meeting on Tuesday 3-24</t>
   </si>
   <si>
@@ -135,9 +132,6 @@
     <t>Contoso Financial - CoPilot Migration #002</t>
   </si>
   <si>
-    <t>Contoso Financial' Engineering team does not have expertise in managing and Governing D365 environments to support the 2 important LOB projects in US Wealth and FCU.</t>
-  </si>
-  <si>
     <t>Jordan Chen</t>
   </si>
   <si>
@@ -177,9 +171,6 @@
     <t>Northwind Medical</t>
   </si>
   <si>
-    <t>ServiceNow Triaging Copilot Studio Agent.</t>
-  </si>
-  <si>
     <t>Waiting on Northwestern for SOW and MSA to be completed.</t>
   </si>
   <si>
@@ -201,12 +192,6 @@
     <t>Fabrikam Government Services</t>
   </si>
   <si>
-    <t>Context on what Public Safety is looking for (we want to keep this straight forward and not overcomplicate things): Code review or code audit services for solutions built on Microsoft technologies, specifically for environments leveraging MS Dynamics, Power Apps, Power Platform components, and associated custom development of plugins. PS’s goal is to validate the quality, robustness, and gather lessons learned on the Phase 2 implementation and to ensure we are following recommended architectural and development practices. Provide more information on : Scope of services offered
-Requirements and materials needed to support an audit
-Estimated timelines and effort
-Cost structure and contracting options within the Government of Canada (i.e. portion that can be financed via Microsoft + others)</t>
-  </si>
-  <si>
     <t>Walk through Draft SOW with Microsoft Team Tuesday.</t>
   </si>
   <si>
@@ -222,14 +207,6 @@
     <t>Contoso Financial - Dynamics Automation #006</t>
   </si>
   <si>
-    <t>exploring potential solutions to multiple inboxes receiving requests from internal and external stakeholders &amp; They receive three types of requests from to their inboxes.
-1.	External emails from other FI’s, customers and law enforcement
-2.	Internal to Contoso Financial a.	External to EFM (i.e. contact center, branch, RM,…) to complete the feedback loop on a case or advise of an event
-b.	Internal to EFM (i.e. hand-offs from one team or Fraud pillar to another) They are looking for a solution to
-1.	Convert external emails to a ticket/case that can be queued and worked.
-2.	Provide a power app form for internal to Contoso Financial partners to create a ticket that can be queued and worked by EFM a.	Internal tickets can have account fields that we can use in conjunction with our fraud book of record to create efficiency.</t>
-  </si>
-  <si>
     <t>Meeting with Engineering and Fraud meeting to discuss working parallel on requirements while governance work is in progress.</t>
   </si>
   <si>
@@ -248,9 +225,6 @@
     <t>Adatum Manufacturing</t>
   </si>
   <si>
-    <t>Volcano Manufacturing faces Project Online retirement in 2026, with potential disruption to current license spend. Modernizing with Planner Premium and D365 Project Operations provides integrated governance and AI‑enabled project/portfolio capabilities.</t>
-  </si>
-  <si>
     <t>Presented Pricing and licensing Waiting on Volcano Manufacturing for feedback.</t>
   </si>
   <si>
@@ -287,9 +261,6 @@
     <t>Adatum Manufacturing - Workstream Digital Front Door #009</t>
   </si>
   <si>
-    <t>Project Operation Quick Start opp for Montreal Project managers currently using Project Desktop.</t>
-  </si>
-  <si>
     <t>Check point meeting with Microsoft team this week.</t>
   </si>
   <si>
@@ -305,9 +276,6 @@
     <t>Adatum Manufacturing - Workstream Process Mining Quick Start #010</t>
   </si>
   <si>
-    <t>Volcano Manufacturing Brazil is evaluating a move from Project Online to Dynamics 365 Project Operations to modernize project visibility, reporting, and governance for complex, custom-engineered projects currently managed through Excel-heavy processes.</t>
-  </si>
-  <si>
     <t>Sync with Microsoft Team and present Proposal and demo to Volcano Manufacturing team.</t>
   </si>
   <si>
@@ -344,9 +312,6 @@
     <t>Fabrikam</t>
   </si>
   <si>
-    <t>Fabrikam faces Project Online retirement in 2026, creating risk around current project management investments. This is a strategic opportunity to modernize with AI-enabled tools and integrated governance through Microsoft Planner Premium and Dynamics 365 Project Operations.</t>
-  </si>
-  <si>
     <t>Meeting with Fabrikam to review SOW, MSA and Data processing document this week.</t>
   </si>
   <si>
@@ -362,9 +327,6 @@
     <t>Volcano Manufacturing</t>
   </si>
   <si>
-    <t>ATS faces Project Online retirement in 2026, creating risk around current project management investments. This is a strategic opportunity to modernize with AI-enabled tools and integrated governance through Microsoft Planner Premium and Dynamics 365 Project Operations.</t>
-  </si>
-  <si>
     <t>Ali Manek new rep from Salesforce just joined to qualify the opportunity with ATS</t>
   </si>
   <si>
@@ -380,9 +342,6 @@
     <t>Tailspin Retail Group</t>
   </si>
   <si>
-    <t>Northwind Traders is pursuing a unified, mobile‑first digital front door using Teams and Copilot Studio to streamline frontline workflows, improve knowledge access, and modernize operational communications across 200,000 colleagues.</t>
-  </si>
-  <si>
     <t>Technical deep dive with Northwind Traders team.</t>
   </si>
   <si>
@@ -401,16 +360,6 @@
     <t>Woodgrove Utilities</t>
   </si>
   <si>
-    <t>Client: Vistra Opportunity Type: Advisory + Enablement (Power Platform &amp; Copilot) Drivers: Rapid business-led adoption, need for scalable governance, executive sponsorship Requested Support:
-Governance design (Power Platform &amp; Copilot)
-Enablement model refinement and scaling
-Optional process intelligence positioning
-Engagement Shape:
-Short, focused advisory engagement
-Two parallel streams (Governance + Enablement)
-Strong alignment with both IT and business stakeholders</t>
-  </si>
-  <si>
     <t>Client meeting to discuss enablement and governance proposal</t>
   </si>
   <si>
@@ -426,9 +375,6 @@
     <t>Contoso Financial 7</t>
   </si>
   <si>
-    <t>Contoso Financial 7 faces Project Online retirement in 2026, risking disruption to $500K annual license spend. This is a strategic opportunity to modernize project management with AI-enabled tools and integrated governance through Microsoft Planner Premium and Dynamics 365 Project Operations.</t>
-  </si>
-  <si>
     <t>Check in meeting with Microsoft Rep Lydia to track progress .</t>
   </si>
   <si>
@@ -444,9 +390,6 @@
     <t>Volcano Manufacturing 5</t>
   </si>
   <si>
-    <t>Textron faces the 2026 retirement of Project Online, creating risk to project/portfolio continuity and compliance. The migration is a timely opportunity to modernize with Planner Premium and D365 Project Operations and adopt AI‑assisted governance.</t>
-  </si>
-  <si>
     <t>Microsoft influencing no RFP -- standing by for intro. Microsoft to present ECIF in 2 weeks and proposal.</t>
   </si>
   <si>
@@ -462,10 +405,6 @@
     <t>Contoso Financial 2</t>
   </si>
   <si>
-    <t>Migration planning from UiPath to Microsoft Power Automate Desktop for LifeLabs, leveraging proprietary migration tool to streamline bot conversion and reduce manual effort.
-2. Opportunity Current Situation</t>
-  </si>
-  <si>
     <t>Meeting with Lifelabs this week to review Complexity report.</t>
   </si>
   <si>
@@ -484,9 +423,6 @@
     <t>Contoso Health</t>
   </si>
   <si>
-    <t>Alithya's workshop delivered Power CAT Workshops to enterprise customers, focusing on enhancing digital presence and customer engagement through AI and Power Platform solutions. This presents a significant opportunity to showcase Alithya's expertise and drive business growth</t>
-  </si>
-  <si>
     <t>Refine proposal with Digital Adoption and review with client next week.</t>
   </si>
   <si>
@@ -502,9 +438,6 @@
     <t>Contoso Financial 5</t>
   </si>
   <si>
-    <t>Tangerine is evaluating D365 Sales Premium to replace manual Excel‑based sales processes. Initial rollout for 30 users with scale to 250. Seeking rapid deployment and enablement supported by Alithya under existing MSA.</t>
-  </si>
-  <si>
     <t>Tangerine confirming funding.</t>
   </si>
   <si>
@@ -518,9 +451,6 @@
   </si>
   <si>
     <t>Adatum Solutions</t>
-  </si>
-  <si>
-    <t>Qty of Proj Online Essentials is 346, and P3 (which includes Planner &amp; Proj Online) is 360. We'll get you going with an NDA for them, so that you can learn more and see reverse demo.</t>
   </si>
   <si>
     <t>STEP 3 – Migration Options Review Session
@@ -540,9 +470,6 @@
     <t>Volcano Manufacturing 2</t>
   </si>
   <si>
-    <t>Johnson Controls faces Project Online retirement in 2026, risking disruption to their annual Project Online license spend. This is a strategic opportunity to modernize project management with AI-enabled tools and integrated governance through Microsoft Planner Premium and Dynamics 365 Project Operations.</t>
-  </si>
-  <si>
     <t>Standing by from Microsoft to engage</t>
   </si>
   <si>
@@ -558,9 +485,6 @@
     <t>Contoso</t>
   </si>
   <si>
-    <t>Contoso faces Project Online retirement in 2026, creating risk around current project management investments. This is a strategic opportunity to modernize with AI-enabled tools and integrated governance through Microsoft Planner Premium and Dynamics 365 Project Operations.</t>
-  </si>
-  <si>
     <t>Reached out to AE from Microsoft to confirm opp and AI Business Solutions seller.</t>
   </si>
   <si>
@@ -576,9 +500,6 @@
     <t>Northwind Traders</t>
   </si>
   <si>
-    <t>Home Hardware has a significant opportunity to enhance its dealer support operations by implementing process intelligence and automation. By leveraging Microsoft’s Power Platform and AI technologies, the company aims to transform its support model from reactive to proactive, improving resolution times, preventing bottlenecks, and enhancing the overall support experience for its independent dealers</t>
-  </si>
-  <si>
     <t>Need SOW like Northwestern for Home Hardware -- Copy paste.</t>
   </si>
   <si>
@@ -600,9 +521,6 @@
     <t>Fabrikam Tech</t>
   </si>
   <si>
-    <t>Moneris is looking for a replacement system for a home built Integrated Solutions Tracking application. This application is used for the onboarding of a new client and configurtation and distribution of a device/integration channel for this client.</t>
-  </si>
-  <si>
     <t>Waiting on Moneris given the org changes for this application Re platform decision.</t>
   </si>
   <si>
@@ -618,11 +536,6 @@
     <t>Fabrikam Government Services - Workstream Agent Accelerator #026</t>
   </si>
   <si>
-    <t>This opportunity originated through Pascale Laroche at Microsoft and targets Fabrikam Government Services as they launch a time-sensitive pilot initiative for the Deputy Minister’s Office focused on modernizing departmental tasking. The customer’s current tasking workflow is spread across multiple disconnected tools and channels, including SharePoint lists, Planner, GC Docs, email, Excel files, and attachments. This fragmentation is contributing to inconsistent execution, loss of comments and context, limited auditability, and a high administrative burden in a process that must support senior leadership responsiveness. [Task Autom...initiative | Word], [TA 11 - 't...s 05012025 | PDF]
-Public Safety established a Corporate Secretariat function to coordinate departmental taskings supporting multiple Deputy Ministers and Ministers, and the operating environment now requires a more unified, traceable, and scalable approach to intake, triage, assignment, drafting, review, packaging, and archiving. The opportunity is to help Public Safety move from manual, disconnected activities to a cohesive end-to-end task management capability, anchored by a centralized intake and tracking experience, workflow automation, stronger governance, and improved transparency for stakeholders. [TA 11 - 't...s 05012025 | PDF]
-The engagement is expected to begin with a discovery phase to validate architecture and implementation path, assess the current SharePoint/Power Apps pilot and how it can evolve responsibly, and define workflow patterns that accommodate varying task types and multi-tier approvals (e.g., Director, DG, ADM, Deputy Minister). The target scale includes approximately ~500 task creators and up to ~2000 recipients, requiring careful attention to scalability, audit trails, and licensing implications</t>
-  </si>
-  <si>
     <t>Review Solution Design with Ram then schedule review meeting with Marco/Pascale from Microsoft</t>
   </si>
   <si>
@@ -635,9 +548,6 @@
     <t>Volcano Manufacturing 2 - Workstream Code Review #027</t>
   </si>
   <si>
-    <t>Copilot Studio Agent Accelerator proposal</t>
-  </si>
-  <si>
     <t>Meet with Champion manager in New Year to review the proposal for Process to Agent Accelerator.</t>
   </si>
   <si>
@@ -656,9 +566,6 @@
     <t>Fabrikam Power</t>
   </si>
   <si>
-    <t>The Fabrikam Power (IESO) is preparing to issue an RFP for the implementation of Microsoft Dynamics 365 Customer Service (D365 CS) in January. As Ontario’s Crown corporation responsible for managing the province’s electricity system and wholesale market, IESO is seeking to modernize its customer engagement and service delivery capabilities. The organization oversees real-time grid operations, market administration, and long-term planning, serving over 5.3 million consumers and handling $23 billion in annual transactions. With the ongoing Market Renewal Program (MRP) and increasing demand for transparency, efficiency, and reliability, IESO recognizes the need for a robust CRM platform to support its evolving business processes. This opportunity centers on delivering a scalable, secure, and integrated D365 CS solution that aligns with IESO’s strategic goals, regulatory requirements, and commitment to customer-centric service. The successful implementation will empower IESO to streamline case management, enhance stakeholder communications, and drive operational excellence across its enterprise.</t>
-  </si>
-  <si>
     <t>Follow up with Mokhtar on RFP release date.</t>
   </si>
   <si>
@@ -671,9 +578,6 @@
     <t>Contoso Financial - Workstream Modernization #029</t>
   </si>
   <si>
-    <t>Contoso Financial is exploring AI-led modernization of its Contact Center to improve agent efficiency, reduce handle time, and enhance customer experience using Copilot and Azure AI capabilities aligned to enterprise banking needs.</t>
-  </si>
-  <si>
     <t>Follow up with Michael She now that Dataverse is unblocked.</t>
   </si>
   <si>
@@ -713,9 +617,6 @@
     <t>Contoso Energy</t>
   </si>
   <si>
-    <t>Had blue prism did not work for them have Power Automate kind of working need foundational plus advance Power Automate workloads. Working with Tony Zettel and Ori Fishler and Chris Bain SSP from Microsoft</t>
-  </si>
-  <si>
     <t>Meet with Tony to discuss next steps.</t>
   </si>
   <si>
@@ -734,25 +635,6 @@
     <t>Contoso Financial 4</t>
   </si>
   <si>
-    <t>Power Platform COE Engagement
-How do we build a better Governance framework.
-Some issues with Default Environment. Power Pages POC
-POC possible
-Like to include their developers
-Would be an externally facing site. Current priority is Governance
-DLP review
-Classification of environments
-Have a target to get people out of the default 38 PowerApps that are custom built to support the organization. Deployment Pipelines ALM
-Are we doing it the best way or is their a better way. Priority List
-Governance Framework
-Environment Framework
-Security Workshop.
-Learning session on the new Admin Center.
-ALM and Pipelines
-Default Env Monitoring
-Power Pages POC</t>
-  </si>
-  <si>
     <t>Followed up awaiting to hear back from OTPP.</t>
   </si>
   <si>
@@ -771,9 +653,6 @@
     <t>Adatum</t>
   </si>
   <si>
-    <t>Farber seeks a strategic partner to drive an integrated enterprise transformation, redesigning processes, org model, data foundations, and modernizing Dynamics 365/Power Platform to build a scalable, efficient, client‑centric operation.</t>
-  </si>
-  <si>
     <t>Reconnect with Farber in 2 months to check in on initiative.</t>
   </si>
   <si>
@@ -789,9 +668,6 @@
     <t>Fabrikam Healthcare</t>
   </si>
   <si>
-    <t>Opportunity to partner with Oracle team on Cost of Care solution and Process Mining</t>
-  </si>
-  <si>
     <t>CIO retiring. need to move out til fall to pick this back up iwth Corey</t>
   </si>
   <si>
@@ -816,9 +692,6 @@
     <t>Contoso Public Sector</t>
   </si>
   <si>
-    <t>RFP for CRM Contoso Public Sector.</t>
-  </si>
-  <si>
     <t>Awarded -- Complete MSA and sign back by Dec 31st.</t>
   </si>
   <si>
@@ -834,9 +707,6 @@
     <t>Volcano Manufacturing 4</t>
   </si>
   <si>
-    <t>Volcano Manufacturing 4 is exploring AI and Copilot adoption but faces strict ROI requirements from its private equity owners. ERP replacement is off the table, yet inefficiencies persist across SAP, QAD, ProfitKey, and custom shop-floor systems. The proposed engagement leverages Microsoft-funded process mining to uncover automation opportunities, quantify ROI, and identify high-impact use cases for Copilot and Power Platform. This approach provides a clear, data-driven roadmap for AI adoption without major system changes.</t>
-  </si>
-  <si>
     <t>Send Volcano Manufacturing 4 updated proposal with updated MS funding</t>
   </si>
   <si>
@@ -852,9 +722,6 @@
     <t>Fourth Coffee Financial</t>
   </si>
   <si>
-    <t>Copilot Studio Accelerator offer</t>
-  </si>
-  <si>
     <t>Check in meeting scheduled for Dec 12th to position our Copilot Accelerator offer.</t>
   </si>
   <si>
@@ -873,9 +740,6 @@
     <t>Woodgrove Financial</t>
   </si>
   <si>
-    <t>John Hancock Finance is exploring AI adoption aligned to Manulife’s 2026 direction. Microsoft initiated an enablement path to clarify Copilot for M365 vs. Copilot Studio and identify Finance-focused AI use cases leading to a potential PoC.</t>
-  </si>
-  <si>
     <t>Connect with Lydia Microsoft SSP on next steps. work with Nyell to understand MCI funding availability.</t>
   </si>
   <si>
@@ -888,9 +752,6 @@
     <t>Tailspin Retail Group - Workstream Code Review #041</t>
   </si>
   <si>
-    <t>Northwind Traders is moving from Appian, Moveworks and Blue Prism to Power Platform as part of tools consolidation / renewal propsoal.</t>
-  </si>
-  <si>
     <t>Follow up with Northwind Traders on where this sits in the 2026 priorities and waiting to hear back.</t>
   </si>
   <si>
@@ -906,9 +767,6 @@
     <t>Contoso Manufacturing</t>
   </si>
   <si>
-    <t>Copilot Studio Agent Accelerator</t>
-  </si>
-  <si>
     <t>Touch point meeting in May.</t>
   </si>
   <si>
@@ -927,9 +785,6 @@
     <t>Northwind Importers</t>
   </si>
   <si>
-    <t>Launch Autonomous Copilot Studio Agent</t>
-  </si>
-  <si>
     <t>Meet with Jeramie / Thomas power Chicago Workshop to review SOW on Copilto Studio Agent.</t>
   </si>
   <si>
@@ -945,9 +800,6 @@
     <t>Tailspin Retail Group - Workstream Migration #044</t>
   </si>
   <si>
-    <t>Enhance Northwind Traders’s Coplan App by adding a secure Power Pages portal for external consultants to directly update assigned records, improving efficiency and data quality.</t>
-  </si>
-  <si>
     <t>Key Business stakeholder on leave for at least a month. Project on hold until he gets back. Follow up end of feb.</t>
   </si>
   <si>
@@ -966,9 +818,6 @@
     <t>Contoso Financial 3</t>
   </si>
   <si>
-    <t>Engage Manulife ETS Innovation team to showcase Alethea’s agentic AI and process mining capabilities, aiming to support their 3–5 year strategy through pilot projects and knowledge transfer.</t>
-  </si>
-  <si>
     <t>Meeting schedule with ETS Innovations lead to talk about next steps. John Hancock MSA in place.</t>
   </si>
   <si>
@@ -984,9 +833,6 @@
     <t>Tailspin Retail Group - Workstream Governance #046</t>
   </si>
   <si>
-    <t>Automate a secure, accessible change log for six critical tables in the Coplan app, enabling non-licensed users to view updates, improving transparency and reducing manual reporting.</t>
-  </si>
-  <si>
     <t>301a32a8-930e-4f23-a6f4-111ce156a27b</t>
   </si>
   <si>
@@ -996,9 +842,6 @@
     <t>Tailspin Retail Group - Workstream AI Pilot #047</t>
   </si>
   <si>
-    <t>RFQ portal Vendor updates plus a security engagement with Glitch secure</t>
-  </si>
-  <si>
     <t>Prepare CR and send to Senthil for entry into field glass.</t>
   </si>
   <si>
@@ -1014,9 +857,6 @@
     <t>World Wide Importers</t>
   </si>
   <si>
-    <t>Copilot Studio Agent Accelerator offer</t>
-  </si>
-  <si>
     <t>Customer has gone dark following up again..</t>
   </si>
   <si>
@@ -1032,9 +872,6 @@
     <t>Volcano Manufacturing 2 - Workstream Contact Center Upgrade #049</t>
   </si>
   <si>
-    <t>JCI wants to migrate some UI Autonomous Bots to Power Automate Process to save $</t>
-  </si>
-  <si>
     <t>Complete MSA with Project Ops opportunity.</t>
   </si>
   <si>
@@ -1050,9 +887,6 @@
     <t>Contoso Technology</t>
   </si>
   <si>
-    <t>Managed service F&amp;O Hydrosolutions.</t>
-  </si>
-  <si>
     <t>Introduction meeting with Microsoft team to Yuri in Montreal hydrosolutions.</t>
   </si>
   <si>
@@ -1065,9 +899,6 @@
     <t>Contoso Financial - Workstream Digital Front Door #051</t>
   </si>
   <si>
-    <t>Deploy M365 Copilot and Copilot Studio to liberate human capacity across Contoso Financial</t>
-  </si>
-  <si>
     <t>Proposal to unblock Dataverse being sent to Contoso Financial this week to unblock this opp.</t>
   </si>
   <si>
@@ -1083,9 +914,6 @@
     <t>Contoso 2</t>
   </si>
   <si>
-    <t>Core Plus Flex Delivery Model: We aligned on implementing a delivery structure with a stable core team (architects, program managers) and a flexible team to manage backlog fluctuations. The model will incorporate compliance-specific activities tailored for regulated life sciences environments.</t>
-  </si>
-  <si>
     <t>check back in with Champion once they have solved their AI Literacy.</t>
   </si>
   <si>
@@ -1101,9 +929,6 @@
     <t>Contoso Financial - Workstream RPA Consolidation #053</t>
   </si>
   <si>
-    <t>Migration of share mailboxes plus introduction of AI into the solution at scale with Agents</t>
-  </si>
-  <si>
     <t>Complete Phase 1.</t>
   </si>
   <si>
@@ -1149,9 +974,6 @@
     <t>Northwind Digital - Workstream Managed Services #056</t>
   </si>
   <si>
-    <t>Managed support agreement</t>
-  </si>
-  <si>
     <t>Meeting with Contoso Technology Wednesday to get an update on this proposal.</t>
   </si>
   <si>
@@ -1164,9 +986,6 @@
     <t>Contoso Financial - Workstream Modernization #057</t>
   </si>
   <si>
-    <t>Celonis is expiring in Fall. Looking at PM &amp; recently attended a meeting regarding data mining in process; use Celonis which is more expensive than Process Mining.</t>
-  </si>
-  <si>
     <t>Weekly check points with GIo.</t>
   </si>
   <si>
@@ -1182,9 +1001,6 @@
     <t>Woodgrove</t>
   </si>
   <si>
-    <t>The opportunity at Woodgrove is centered around enhancing their Power Platform governance and operationalizing the knowledge gained from the Power CAT workshop. The internal champion, Heidy Nuevo, is driving the initiative with strong engagement and coordination. The economic buyer, Michael Jimerson, VP of IT, will authorize funding and is crucial for the project's approval.</t>
-  </si>
-  <si>
     <t>Review Use case and 2026 funding with First service third week of March.</t>
   </si>
   <si>
@@ -1200,9 +1016,6 @@
     <t>Northwind Digital - Workstream Enablement #059</t>
   </si>
   <si>
-    <t>Phase 0 (Commerce) focuses on a lift‑and‑shift from Salesforce and is defined as a standalone scope of work. It includes sales order notifications and the tracking of customer entitlements and subscriptions, which are currently managed in Salesforce, and will be refactored as part of the B2B flow with an emphasis on process improvement. In parallel, this phase delivers improved CRM–Finance &amp; Operations (F&amp;O) integration by enhancing prioritized integration touchpoints to enable easier data access, stronger reporting outcomes, and a more consistent end‑user experience, without attempting a full ERP redesign.</t>
-  </si>
-  <si>
     <t>Circle back post Salesforce migration.</t>
   </si>
   <si>
@@ -1248,7 +1061,163 @@
     <t>Probability</t>
   </si>
   <si>
-    <t>PIPELINE TEST – SHOULD SHOW IN PROD</t>
+    <t>CRM platform upgrade from version 7.5 to 8.3 on-premises deployment</t>
+  </si>
+  <si>
+    <t>Tech division lacks skills to manage enterprise environments for 3 key business initiatives in Regional Operations and Corporate Services.</t>
+  </si>
+  <si>
+    <t>DEMO ENTRY – FOR TESTING PURPOSES</t>
+  </si>
+  <si>
+    <t>IT helpdesk routing automation tool deployment.</t>
+  </si>
+  <si>
+    <t>Government agency seeks code audit for enterprise solutions on cloud tech stack. Goals: validate quality, document best practices from prior deployment. Need info on audit scope, requirements, timelines, pricing options including vendor co-funding.</t>
+  </si>
+  <si>
+    <t>Evaluating solutions for unified inbox management across departments. Need to convert external inquiries to trackable cases, create internal request forms, and link records to operational systems for streamlined case handling.</t>
+  </si>
+  <si>
+    <t>Corp ABC faces legacy system sunset in 2027. Risk to current software investments. Opportunity to upgrade with modern planning tools and cloud-based project management featuring AI capabilities.</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Quick-start project management deployment for regional team leads currently using desktop applications.</t>
+  </si>
+  <si>
+    <t>Latin America division evaluating shift from legacy tools to cloud project management for better visibility and governance on complex engineering projects currently tracked via spreadsheets.</t>
+  </si>
+  <si>
+    <t>Enterprise Corp faces legacy tool retirement next year. Strategic modernization opportunity with AI-enabled project tools and integrated governance through cloud-based planning solutions.</t>
+  </si>
+  <si>
+    <t>Global Industries faces system sunset next year. Strategic chance to upgrade project management with AI tools and unified governance through modern cloud planning platform.</t>
+  </si>
+  <si>
+    <t>Regional Retail seeks unified mobile-first employee portal using collaboration tools to streamline frontline operations, boost knowledge sharing, and modernize communications for 150K staff.</t>
+  </si>
+  <si>
+    <t>Client: Energy Co. Type: Strategy + Training. Drivers: Fast organic growth, governance needs, exec support. Scope: Platform governance, enablement scaling, process analytics. Format: Focused advisory with parallel workstreams.</t>
+  </si>
+  <si>
+    <t>Banking Group 7 faces legacy retirement in 2027, risking $400K annual costs. Chance to modernize with AI tools and unified governance via cloud planning and operations platform.</t>
+  </si>
+  <si>
+    <t>Industrial Corp faces 2027 legacy system end-of-life, risking continuity. Migration enables modern planning tools with AI governance and integrated operations management.</t>
+  </si>
+  <si>
+    <t>RPA migration from third-party tool to enterprise automation platform, using proprietary converter to accelerate bot transition and minimize manual rework.</t>
+  </si>
+  <si>
+    <t>Consulting firm delivered platform workshops to enterprise clients, focusing on digital transformation and engagement via AI solutions. Key opportunity to demonstrate expertise and expand revenue.</t>
+  </si>
+  <si>
+    <t>Banking firm evaluating CRM Premium for 25-user pilot scaling to 200. Seeking fast deployment with partner support under existing agreement.</t>
+  </si>
+  <si>
+    <t>License count: 280 Standard, 300 Premium. Planning NDA for detailed discovery and product demonstration session.</t>
+  </si>
+  <si>
+    <t>Industrial Corp faces legacy system retirement next year, risking license costs. Strategic modernization with AI planning tools and integrated governance through cloud operations platform.</t>
+  </si>
+  <si>
+    <t>Enterprise Corp faces legacy retirement next year. Strategic chance to modernize with AI tools and unified governance via cloud planning and project operations.</t>
+  </si>
+  <si>
+    <t>Retail chain opportunity to enhance dealer support via process intelligence and automation. Using platform AI to shift from reactive to proactive support, cutting resolution times for independent partners.</t>
+  </si>
+  <si>
+    <t>Payment processor needs replacement for custom-built tracking app used for client onboarding and device channel configuration/distribution.</t>
+  </si>
+  <si>
+    <t>Government agency pilot for executive task management modernization. Current workflow fragmented across lists, docs, email. Need unified intake, tracking, workflow automation for ~400 creators and 1500 recipients.</t>
+  </si>
+  <si>
+    <t>AI Assistant Rapid Deployment proposal</t>
+  </si>
+  <si>
+    <t>Energy Authority issuing RFP for CRM implementation. Crown corp managing provincial grid and $18B market seeks modern customer service platform for 4.5M consumers with compliance and transparency goals.</t>
+  </si>
+  <si>
+    <t>Banking Corp exploring AI-driven contact center modernization to boost agent productivity, reduce handling time, and improve CX using assistant and cloud AI aligned to enterprise needs.</t>
+  </si>
+  <si>
+    <t>Previous RPA tool failed. Now using enterprise automation with basic implementation. Need foundational plus advanced workflow training. Coordinating with vendor specialists.</t>
+  </si>
+  <si>
+    <t>Platform COE initiative: governance framework, environment classification, DLP review. 32 custom apps to migrate from default. Priorities: admin training, pipelines, environment monitoring, external portal POC.</t>
+  </si>
+  <si>
+    <t>Consulting firm seeks strategic partner for enterprise transformation: process redesign, org model, data foundations, and platform modernization for scalable client-focused operations.</t>
+  </si>
+  <si>
+    <t>Partnership opportunity with ERP team on healthcare cost solution and process analytics</t>
+  </si>
+  <si>
+    <t>RFP for CRM implementation at government agency.</t>
+  </si>
+  <si>
+    <t>Manufacturing Co exploring AI adoption with strict PE-mandated ROI targets. ERP change not viable, but inefficiencies exist across multiple systems. Vendor-funded process mining to find automation opportunities and AI use cases.</t>
+  </si>
+  <si>
+    <t>AI Assistant Accelerator offering</t>
+  </si>
+  <si>
+    <t>Insurance division exploring AI adoption per parent company 2027 strategy. Vendor enabling clarity on assistant options and identifying finance-focused AI use cases for potential pilot.</t>
+  </si>
+  <si>
+    <t>Distribution Corp migrating from legacy RPA and workflow tools to unified automation platform as part of vendor consolidation initiative.</t>
+  </si>
+  <si>
+    <t>AI Assistant Rapid Deployment</t>
+  </si>
+  <si>
+    <t>Deploy Autonomous AI Assistant Agent</t>
+  </si>
+  <si>
+    <t>Enhance project tracking app with secure external portal for contractors to update assigned records, improving efficiency and data accuracy.</t>
+  </si>
+  <si>
+    <t>Partner with Innovation team to demo AI agent and process mining capabilities, supporting 4-year strategy via pilots and knowledge transfer.</t>
+  </si>
+  <si>
+    <t>Build automated change log for 5 key tables in project app, letting view-only users see updates while cutting manual reporting overhead.</t>
+  </si>
+  <si>
+    <t>Vendor portal updates plus security assessment engagement</t>
+  </si>
+  <si>
+    <t>AI Assistant Rapid Deployment offering</t>
+  </si>
+  <si>
+    <t>Corp wants to migrate autonomous bots to enterprise automation to reduce costs</t>
+  </si>
+  <si>
+    <t>Managed services for ERP implementation at water solutions company.</t>
+  </si>
+  <si>
+    <t>Deploy AI assistants across enterprise to free up staff capacity at Banking Corp</t>
+  </si>
+  <si>
+    <t>Flexible delivery model with stable core team (architects, PMs) plus flex resources for backlog. Includes compliance activities for regulated industries.</t>
+  </si>
+  <si>
+    <t>Email system migration plus AI agent introduction at enterprise scale</t>
+  </si>
+  <si>
+    <t>Managed support contract</t>
+  </si>
+  <si>
+    <t>Process analytics vendor contract expiring in autumn. Evaluating alternatives; attended data mining demo. Current tool more costly than competing options.</t>
+  </si>
+  <si>
+    <t>Opportunity centers on platform governance and operationalizing workshop learnings. Internal champion driving initiative with exec buyer VP of Technology authorizing funding.</t>
+  </si>
+  <si>
+    <t>Phase 0: CRM migration from legacy system as standalone scope. Includes order notifications, subscription tracking with process improvement. Parallel effort improves CRM-ERP integration for better reporting and UX.</t>
   </si>
 </sst>
 </file>
@@ -1315,6 +1284,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1728,7 +1701,7 @@
         <v>13</v>
       </c>
       <c r="O1" t="s">
-        <v>391</v>
+        <v>340</v>
       </c>
       <c r="P1" t="s">
         <v>14</v>
@@ -1763,10 +1736,10 @@
         <v>22</v>
       </c>
       <c r="F2" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="H2" s="4">
         <v>46107.833333333343</v>
@@ -1778,13 +1751,13 @@
         <v>177000</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N2" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="O2" s="6">
         <f t="shared" ref="O2:O33" si="0">IF(S2="","",VALUE(LEFT(S2,FIND("%",S2)-1)))</f>
@@ -1797,33 +1770,33 @@
         <v>46105.541342592587</v>
       </c>
       <c r="R2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="S2" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:20" ht="72.900000000000006" customHeight="1">
       <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="C3" s="2">
         <v>46109.622002314813</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>33</v>
+        <v>342</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H3" s="4">
         <v>46107.833333333343</v>
@@ -1835,13 +1808,13 @@
         <v>90100</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="M3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N3" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="O3" s="6">
         <f t="shared" si="0"/>
@@ -1854,33 +1827,33 @@
         <v>46109.455335648148</v>
       </c>
       <c r="R3" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S3" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:20" ht="409.6" customHeight="1">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C4" s="2">
         <v>46103.914571759262</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>343</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>392</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>40</v>
       </c>
       <c r="H4" s="4">
         <v>46107.833333333343</v>
@@ -1892,13 +1865,13 @@
         <v>2391000</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N4" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="O4" s="6">
         <f t="shared" si="0"/>
@@ -1911,30 +1884,30 @@
         <v>46103.74790509259</v>
       </c>
       <c r="S4" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:20" ht="29.15" customHeight="1">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C5" s="2">
         <v>46103.914872685193</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>48</v>
       </c>
       <c r="H5" s="4">
         <v>46121.833333333343</v>
@@ -1946,13 +1919,13 @@
         <v>96300</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="M5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N5" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="N5" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="O5" s="6">
         <f t="shared" si="0"/>
@@ -1965,33 +1938,33 @@
         <v>46103.748206018521</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="S5" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:20" ht="409.6" customHeight="1">
       <c r="A6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C6" s="2">
         <v>46109.880787037036</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>55</v>
+        <v>345</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="H6" s="4">
         <v>46107.833333333343</v>
@@ -2003,10 +1976,10 @@
         <v>51800</v>
       </c>
       <c r="M6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N6" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="N6" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="O6" s="6">
         <f t="shared" si="0"/>
@@ -2019,30 +1992,30 @@
         <v>46109.714120370372</v>
       </c>
       <c r="S6" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:20" ht="409.6" customHeight="1">
       <c r="A7" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C7" s="2">
         <v>46105.599699074082</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>61</v>
+        <v>346</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="H7" s="4">
         <v>46107.833333333343</v>
@@ -2054,13 +2027,13 @@
         <v>129000</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="M7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N7" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="N7" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="O7" s="6">
         <f t="shared" si="0"/>
@@ -2073,33 +2046,33 @@
         <v>46105.433032407411</v>
       </c>
       <c r="R7" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="S7" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:20" ht="116.6" customHeight="1">
       <c r="A8" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C8" s="2">
         <v>46109.750381944446</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>68</v>
+        <v>347</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="H8" s="4">
         <v>46107.833333333343</v>
@@ -2111,10 +2084,10 @@
         <v>128000</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O8" s="6">
         <f t="shared" si="0"/>
@@ -2127,30 +2100,33 @@
         <v>46109.583715277768</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:20">
       <c r="A9" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C9" s="2">
         <v>46109.621111111112</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>348</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="H9" s="4">
         <v>46114.833333333343</v>
@@ -2162,10 +2138,10 @@
         <v>272000</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O9" s="6">
         <f t="shared" si="0"/>
@@ -2178,30 +2154,30 @@
         <v>46109.454444444447</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10" spans="1:20" ht="43.75" customHeight="1">
       <c r="A10" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="C10" s="2">
         <v>46104.021504629629</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>81</v>
+        <v>349</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="H10" s="4">
         <v>46107.833333333343</v>
@@ -2213,10 +2189,10 @@
         <v>81900</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O10" s="6">
         <f t="shared" si="0"/>
@@ -2229,30 +2205,30 @@
         <v>46103.854837962957</v>
       </c>
       <c r="S10" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:20" ht="116.6" customHeight="1">
       <c r="A11" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="C11" s="2">
         <v>46104.028715277767</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>87</v>
+        <v>350</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="H11" s="4">
         <v>46107.833333333343</v>
@@ -2264,10 +2240,10 @@
         <v>121000</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="O11" s="6">
         <f t="shared" si="0"/>
@@ -2280,27 +2256,30 @@
         <v>46103.86204861111</v>
       </c>
       <c r="S11" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:20">
       <c r="A12" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C12" s="2">
         <v>46091.595057870371</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>93</v>
+        <v>85</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>348</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="H12" s="4">
         <v>46079.791666666657</v>
@@ -2312,13 +2291,13 @@
         <v>69800</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O12" s="6">
         <f t="shared" si="0"/>
@@ -2331,30 +2310,30 @@
         <v>46091.428391203714</v>
       </c>
       <c r="S12" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:20" ht="145.75" customHeight="1">
       <c r="A13" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C13" s="2">
         <v>46109.74454861111</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>100</v>
+        <v>351</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="H13" s="4">
         <v>46107.833333333343</v>
@@ -2366,10 +2345,10 @@
         <v>114000</v>
       </c>
       <c r="M13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N13" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="N13" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="O13" s="6">
         <f t="shared" si="0"/>
@@ -2382,30 +2361,30 @@
         <v>46109.577881944453</v>
       </c>
       <c r="S13" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:20" ht="145.75" customHeight="1">
       <c r="A14" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="C14" s="2">
         <v>46092.730868055558</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>106</v>
+        <v>352</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="H14" s="4">
         <v>46100.833333333343</v>
@@ -2417,10 +2396,10 @@
         <v>137000</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O14" s="6">
         <f t="shared" si="0"/>
@@ -2433,30 +2412,30 @@
         <v>46092.564201388886</v>
       </c>
       <c r="S14" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:20" ht="116.6" customHeight="1">
       <c r="A15" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="C15" s="2">
         <v>46109.622673611113</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>112</v>
+        <v>353</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="H15" s="4">
         <v>46107.833333333343</v>
@@ -2468,13 +2447,13 @@
         <v>871000</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O15" s="6">
         <f t="shared" si="0"/>
@@ -2487,33 +2466,33 @@
         <v>46109.456006944441</v>
       </c>
       <c r="R15" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S15" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" spans="1:20" ht="364.3" customHeight="1">
       <c r="A16" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="C16" s="2">
         <v>46085.81453703704</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>119</v>
+        <v>354</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="H16" s="4">
         <v>46090.833333333343</v>
@@ -2525,10 +2504,10 @@
         <v>148000</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O16" s="6">
         <f t="shared" si="0"/>
@@ -2541,30 +2520,30 @@
         <v>46085.606203703697</v>
       </c>
       <c r="S16" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:19" ht="145.75" customHeight="1">
       <c r="A17" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C17" s="2">
         <v>46092.924409722233</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>125</v>
+        <v>355</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="H17" s="4">
         <v>46044.791666666657</v>
@@ -2576,10 +2555,10 @@
         <v>165000</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O17" s="6">
         <f t="shared" si="0"/>
@@ -2592,30 +2571,30 @@
         <v>46092.757743055547</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="131.15" customHeight="1">
       <c r="A18" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
       <c r="C18" s="2">
         <v>46109.623738425929</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>131</v>
+        <v>356</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="H18" s="4">
         <v>46100.833333333343</v>
@@ -2627,10 +2606,10 @@
         <v>165000</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O18" s="6">
         <f t="shared" si="0"/>
@@ -2643,30 +2622,30 @@
         <v>46109.457071759258</v>
       </c>
       <c r="S18" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" spans="1:19" ht="102" customHeight="1">
       <c r="A19" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="C19" s="2">
         <v>46084.939201388886</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>137</v>
+        <v>357</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>138</v>
+        <v>123</v>
       </c>
       <c r="H19" s="4">
         <v>46079.791666666657</v>
@@ -2678,13 +2657,13 @@
         <v>42900</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O19" s="6">
         <f t="shared" si="0"/>
@@ -2697,30 +2676,30 @@
         <v>46084.730868055558</v>
       </c>
       <c r="S19" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:19" ht="145.75" customHeight="1">
       <c r="A20" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
       <c r="C20" s="2">
         <v>46084.652060185188</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>142</v>
+        <v>127</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>143</v>
+        <v>128</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>144</v>
+        <v>358</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>145</v>
+        <v>129</v>
       </c>
       <c r="H20" s="4">
         <v>46093.833333333343</v>
@@ -2732,10 +2711,10 @@
         <v>103000</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O20" s="6">
         <f t="shared" si="0"/>
@@ -2748,30 +2727,30 @@
         <v>46084.443726851852</v>
       </c>
       <c r="S20" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:19" ht="116.6" customHeight="1">
       <c r="A21" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>147</v>
+        <v>131</v>
       </c>
       <c r="C21" s="2">
         <v>46092.939074074071</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>149</v>
+        <v>133</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>150</v>
+        <v>359</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="H21" s="4">
         <v>46093.833333333343</v>
@@ -2783,10 +2762,10 @@
         <v>124000</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O21" s="6">
         <f t="shared" si="0"/>
@@ -2799,30 +2778,30 @@
         <v>46092.772407407407</v>
       </c>
       <c r="S21" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" spans="1:19" ht="87.45" customHeight="1">
       <c r="A22" t="s">
-        <v>152</v>
+        <v>135</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>153</v>
+        <v>136</v>
       </c>
       <c r="C22" s="2">
         <v>46097.672395833331</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>154</v>
+        <v>137</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>155</v>
+        <v>138</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>156</v>
+        <v>360</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>157</v>
+        <v>139</v>
       </c>
       <c r="H22" s="4">
         <v>46107.833333333343</v>
@@ -2834,10 +2813,10 @@
         <v>327000</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O22" s="6">
         <f t="shared" si="0"/>
@@ -2850,30 +2829,30 @@
         <v>46097.505729166667</v>
       </c>
       <c r="S22" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" spans="1:19" ht="160.30000000000001" customHeight="1">
       <c r="A23" t="s">
-        <v>158</v>
+        <v>140</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>159</v>
+        <v>141</v>
       </c>
       <c r="C23" s="2">
         <v>46092.92459490741</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>160</v>
+        <v>142</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>161</v>
+        <v>143</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>162</v>
+        <v>361</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>163</v>
+        <v>144</v>
       </c>
       <c r="H23" s="4">
         <v>46100.833333333343</v>
@@ -2885,10 +2864,10 @@
         <v>289000</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O23" s="6">
         <f t="shared" si="0"/>
@@ -2901,30 +2880,30 @@
         <v>46092.757928240739</v>
       </c>
       <c r="S23" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="24" spans="1:19" ht="145.75" customHeight="1">
       <c r="A24" t="s">
-        <v>164</v>
+        <v>145</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>165</v>
+        <v>146</v>
       </c>
       <c r="C24" s="2">
         <v>46092.904513888891</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>166</v>
+        <v>147</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>167</v>
+        <v>148</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>168</v>
+        <v>362</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>169</v>
+        <v>149</v>
       </c>
       <c r="H24" s="4">
         <v>46142.833333333343</v>
@@ -2936,10 +2915,10 @@
         <v>107000</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N24" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O24" s="6">
         <f t="shared" si="0"/>
@@ -2952,30 +2931,30 @@
         <v>46092.737847222219</v>
       </c>
       <c r="S24" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="25" spans="1:19" ht="204" customHeight="1">
       <c r="A25" t="s">
-        <v>170</v>
+        <v>150</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>171</v>
+        <v>151</v>
       </c>
       <c r="C25" s="2">
         <v>46092.939305555563</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>172</v>
+        <v>152</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>173</v>
+        <v>153</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>174</v>
+        <v>363</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>175</v>
+        <v>154</v>
       </c>
       <c r="H25" s="4">
         <v>46114.833333333343</v>
@@ -2987,13 +2966,13 @@
         <v>54700</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>176</v>
+        <v>155</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="O25" s="6">
         <f t="shared" si="0"/>
@@ -3006,33 +2985,33 @@
         <v>46092.772638888891</v>
       </c>
       <c r="R25" s="1" t="s">
-        <v>177</v>
+        <v>156</v>
       </c>
       <c r="S25" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="26" spans="1:19" ht="131.15" customHeight="1">
       <c r="A26" t="s">
-        <v>178</v>
+        <v>157</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>179</v>
+        <v>158</v>
       </c>
       <c r="C26" s="2">
         <v>46092.925995370373</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>180</v>
+        <v>159</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>181</v>
+        <v>160</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>182</v>
+        <v>364</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>183</v>
+        <v>161</v>
       </c>
       <c r="H26" s="4">
         <v>46107.833333333343</v>
@@ -3044,13 +3023,13 @@
         <v>293000</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>184</v>
+        <v>162</v>
       </c>
       <c r="M26" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N26" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="N26" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="O26" s="6">
         <f t="shared" si="0"/>
@@ -3063,30 +3042,30 @@
         <v>46092.759328703702</v>
       </c>
       <c r="S26" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:19" ht="409.6" customHeight="1">
       <c r="A27" t="s">
-        <v>185</v>
+        <v>163</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>186</v>
+        <v>164</v>
       </c>
       <c r="C27" s="2">
         <v>46103.988796296297</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>187</v>
+        <v>165</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>188</v>
+        <v>365</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>189</v>
+        <v>166</v>
       </c>
       <c r="H27" s="4">
         <v>46107.833333333343</v>
@@ -3098,10 +3077,10 @@
         <v>179000</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="O27" s="6">
         <f t="shared" si="0"/>
@@ -3114,30 +3093,30 @@
         <v>46103.822129629632</v>
       </c>
       <c r="S27" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="28" spans="1:19" ht="29.15" customHeight="1">
       <c r="A28" t="s">
-        <v>190</v>
+        <v>167</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>191</v>
+        <v>168</v>
       </c>
       <c r="C28" s="2">
         <v>46092.937858796293</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>192</v>
+        <v>169</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>161</v>
+        <v>143</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>193</v>
+        <v>366</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>194</v>
+        <v>170</v>
       </c>
       <c r="H28" s="4">
         <v>46037.791666666657</v>
@@ -3149,13 +3128,13 @@
         <v>62300</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>195</v>
+        <v>171</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O28" s="6">
         <f t="shared" si="0"/>
@@ -3168,30 +3147,30 @@
         <v>46092.771192129629</v>
       </c>
       <c r="S28" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="29" spans="1:19" ht="409.6" customHeight="1">
       <c r="A29" t="s">
-        <v>196</v>
+        <v>172</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>197</v>
+        <v>173</v>
       </c>
       <c r="C29" s="2">
         <v>46109.60869212963</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>198</v>
+        <v>174</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>199</v>
+        <v>175</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>200</v>
+        <v>367</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>201</v>
+        <v>176</v>
       </c>
       <c r="H29" s="4">
         <v>46135.833333333343</v>
@@ -3203,10 +3182,10 @@
         <v>122000</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O29" s="6">
         <f t="shared" si="0"/>
@@ -3219,30 +3198,30 @@
         <v>46109.442025462973</v>
       </c>
       <c r="S29" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30" spans="1:19" ht="116.6" customHeight="1">
       <c r="A30" t="s">
-        <v>202</v>
+        <v>177</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>203</v>
+        <v>178</v>
       </c>
       <c r="C30" s="2">
         <v>46109.610173611109</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>204</v>
+        <v>179</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>205</v>
+        <v>368</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>206</v>
+        <v>180</v>
       </c>
       <c r="H30" s="4">
         <v>46107.833333333343</v>
@@ -3254,10 +3233,10 @@
         <v>90600</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O30" s="6">
         <f t="shared" si="0"/>
@@ -3270,27 +3249,30 @@
         <v>46109.443506944437</v>
       </c>
       <c r="S30" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:19">
       <c r="A31" t="s">
-        <v>207</v>
+        <v>181</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>208</v>
+        <v>182</v>
       </c>
       <c r="C31" s="2">
         <v>46109.610590277778</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>209</v>
+        <v>183</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>348</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>210</v>
+        <v>184</v>
       </c>
       <c r="H31" s="4">
         <v>46107.833333333343</v>
@@ -3302,13 +3284,13 @@
         <v>113000</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="O31" s="6">
         <f t="shared" si="0"/>
@@ -3321,24 +3303,27 @@
         <v>46109.443923611107</v>
       </c>
       <c r="S31" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" spans="1:19">
       <c r="A32" t="s">
-        <v>211</v>
+        <v>185</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>212</v>
+        <v>186</v>
       </c>
       <c r="C32" s="2">
         <v>46109.618576388893</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>213</v>
+        <v>187</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>214</v>
+        <v>188</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>348</v>
       </c>
       <c r="H32" s="4">
         <v>46058.791666666657</v>
@@ -3350,10 +3335,10 @@
         <v>83100</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O32" s="6">
         <f t="shared" si="0"/>
@@ -3366,30 +3351,30 @@
         <v>46109.451909722222</v>
       </c>
       <c r="S32" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="33" spans="1:19" ht="102" customHeight="1">
       <c r="A33" t="s">
-        <v>215</v>
+        <v>189</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>216</v>
+        <v>190</v>
       </c>
       <c r="C33" s="2">
         <v>46109.610821759263</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>217</v>
+        <v>191</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>218</v>
+        <v>192</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>219</v>
+        <v>369</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>220</v>
+        <v>193</v>
       </c>
       <c r="H33" s="4">
         <v>45890.833333333343</v>
@@ -3401,13 +3386,13 @@
         <v>48200</v>
       </c>
       <c r="L33" s="1" t="s">
-        <v>221</v>
+        <v>194</v>
       </c>
       <c r="M33" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O33" s="6">
         <f t="shared" si="0"/>
@@ -3420,30 +3405,30 @@
         <v>46109.444155092591</v>
       </c>
       <c r="S33" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="34" spans="1:19" ht="409.6" customHeight="1">
       <c r="A34" t="s">
-        <v>222</v>
+        <v>195</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>223</v>
+        <v>196</v>
       </c>
       <c r="C34" s="2">
         <v>46109.611643518518</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>224</v>
+        <v>197</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>225</v>
+        <v>198</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>226</v>
+        <v>370</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>227</v>
+        <v>199</v>
       </c>
       <c r="H34" s="4">
         <v>46093.833333333343</v>
@@ -3455,13 +3440,13 @@
         <v>64300</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>228</v>
+        <v>200</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O34" s="6">
         <f t="shared" ref="O34:O61" si="1">IF(S34="","",VALUE(LEFT(S34,FIND("%",S34)-1)))</f>
@@ -3474,30 +3459,30 @@
         <v>46109.444976851853</v>
       </c>
       <c r="S34" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" spans="1:19" ht="116.6" customHeight="1">
       <c r="A35" t="s">
-        <v>229</v>
+        <v>201</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>230</v>
+        <v>202</v>
       </c>
       <c r="C35" s="2">
         <v>46109.619120370371</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>231</v>
+        <v>203</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>232</v>
+        <v>204</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>233</v>
+        <v>371</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>234</v>
+        <v>205</v>
       </c>
       <c r="H35" s="4">
         <v>46138.833333333343</v>
@@ -3509,10 +3494,10 @@
         <v>186000</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O35" s="6">
         <f t="shared" si="1"/>
@@ -3525,30 +3510,30 @@
         <v>46109.452453703707</v>
       </c>
       <c r="S35" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="36" spans="1:19" ht="43.75" customHeight="1">
       <c r="A36" t="s">
-        <v>235</v>
+        <v>206</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>236</v>
+        <v>207</v>
       </c>
       <c r="C36" s="2">
         <v>46109.619351851848</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>237</v>
+        <v>208</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>238</v>
+        <v>209</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>239</v>
+        <v>372</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="H36" s="4">
         <v>46261.833333333343</v>
@@ -3560,10 +3545,10 @@
         <v>42800</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="O36" s="6">
         <f t="shared" si="1"/>
@@ -3576,27 +3561,30 @@
         <v>46109.452685185177</v>
       </c>
       <c r="R36" s="1" t="s">
-        <v>177</v>
+        <v>156</v>
       </c>
       <c r="S36" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="37" spans="1:19">
       <c r="A37" t="s">
-        <v>241</v>
+        <v>211</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>242</v>
+        <v>212</v>
       </c>
       <c r="C37" s="2">
         <v>46109.613946759258</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>67</v>
+        <v>62</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>348</v>
       </c>
       <c r="I37" s="4">
         <v>46293</v>
@@ -3605,10 +3593,10 @@
         <v>200000</v>
       </c>
       <c r="M37" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O37" s="6">
         <f t="shared" si="1"/>
@@ -3621,30 +3609,30 @@
         <v>46109.447280092587</v>
       </c>
       <c r="S37" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="38" spans="1:19" ht="29.15" customHeight="1">
       <c r="A38" t="s">
-        <v>244</v>
+        <v>214</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>245</v>
+        <v>215</v>
       </c>
       <c r="C38" s="2">
         <v>46109.614317129628</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>246</v>
+        <v>216</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>247</v>
+        <v>217</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>248</v>
+        <v>373</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>249</v>
+        <v>218</v>
       </c>
       <c r="H38" s="4">
         <v>46021.791666666657</v>
@@ -3656,10 +3644,10 @@
         <v>242000</v>
       </c>
       <c r="M38" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N38" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O38" s="6">
         <f t="shared" si="1"/>
@@ -3672,30 +3660,30 @@
         <v>46109.447650462957</v>
       </c>
       <c r="S38" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="39" spans="1:19" ht="247.75" customHeight="1">
       <c r="A39" t="s">
-        <v>250</v>
+        <v>219</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>251</v>
+        <v>220</v>
       </c>
       <c r="C39" s="2">
         <v>46109.614664351851</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>252</v>
+        <v>221</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>253</v>
+        <v>222</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>254</v>
+        <v>374</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>255</v>
+        <v>223</v>
       </c>
       <c r="H39" s="4">
         <v>46051.791666666657</v>
@@ -3707,10 +3695,10 @@
         <v>56400</v>
       </c>
       <c r="M39" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N39" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O39" s="6">
         <f t="shared" si="1"/>
@@ -3723,30 +3711,30 @@
         <v>46109.447997685187</v>
       </c>
       <c r="S39" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="40" spans="1:19">
       <c r="A40" t="s">
-        <v>256</v>
+        <v>224</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>257</v>
+        <v>225</v>
       </c>
       <c r="C40" s="2">
         <v>46109.614907407413</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>258</v>
+        <v>226</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>259</v>
+        <v>227</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>260</v>
+        <v>375</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>261</v>
+        <v>228</v>
       </c>
       <c r="H40" s="4">
         <v>46114.833333333343</v>
@@ -3758,13 +3746,13 @@
         <v>34300</v>
       </c>
       <c r="L40" s="1" t="s">
-        <v>262</v>
+        <v>229</v>
       </c>
       <c r="M40" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N40" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O40" s="6">
         <f t="shared" si="1"/>
@@ -3777,30 +3765,30 @@
         <v>46109.448240740741</v>
       </c>
       <c r="S40" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="41" spans="1:19" ht="131.15" customHeight="1">
       <c r="A41" t="s">
-        <v>263</v>
+        <v>230</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>264</v>
+        <v>231</v>
       </c>
       <c r="C41" s="2">
         <v>46109.615717592591</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>265</v>
+        <v>232</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>266</v>
+        <v>233</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>267</v>
+        <v>376</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>268</v>
+        <v>234</v>
       </c>
       <c r="H41" s="4">
         <v>46044.791666666657</v>
@@ -3812,10 +3800,10 @@
         <v>151000</v>
       </c>
       <c r="M41" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N41" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O41" s="6">
         <f t="shared" si="1"/>
@@ -3828,30 +3816,30 @@
         <v>46109.449050925927</v>
       </c>
       <c r="S41" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="42" spans="1:19" ht="58.3" customHeight="1">
       <c r="A42" t="s">
-        <v>269</v>
+        <v>235</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>270</v>
+        <v>236</v>
       </c>
       <c r="C42" s="2">
         <v>46109.616018518522</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>271</v>
+        <v>237</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>272</v>
+        <v>377</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>273</v>
+        <v>238</v>
       </c>
       <c r="H42" s="4">
         <v>46166.833333333343</v>
@@ -3863,13 +3851,13 @@
         <v>192000</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O42" s="6">
         <f t="shared" si="1"/>
@@ -3882,30 +3870,30 @@
         <v>46109.44935185185</v>
       </c>
       <c r="S42" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="43" spans="1:19">
       <c r="A43" t="s">
-        <v>274</v>
+        <v>239</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>275</v>
+        <v>240</v>
       </c>
       <c r="C43" s="2">
         <v>46109.61886574074</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>276</v>
+        <v>241</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>277</v>
+        <v>242</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>278</v>
+        <v>378</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>279</v>
+        <v>243</v>
       </c>
       <c r="H43" s="4">
         <v>46163.833333333343</v>
@@ -3917,13 +3905,13 @@
         <v>86400</v>
       </c>
       <c r="L43" s="1" t="s">
-        <v>280</v>
+        <v>244</v>
       </c>
       <c r="M43" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N43" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O43" s="6">
         <f t="shared" si="1"/>
@@ -3936,30 +3924,30 @@
         <v>46109.452199074083</v>
       </c>
       <c r="S43" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="44" spans="1:19" ht="29.15" customHeight="1">
       <c r="A44" t="s">
-        <v>281</v>
+        <v>245</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>282</v>
+        <v>246</v>
       </c>
       <c r="C44" s="2">
         <v>46109.616550925923</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>283</v>
+        <v>247</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>284</v>
+        <v>248</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>285</v>
+        <v>379</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>286</v>
+        <v>249</v>
       </c>
       <c r="H44" s="4">
         <v>46100.833333333343</v>
@@ -3971,13 +3959,13 @@
         <v>150000</v>
       </c>
       <c r="L44" s="1" t="s">
-        <v>287</v>
+        <v>250</v>
       </c>
       <c r="M44" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N44" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O44" s="6">
         <f t="shared" si="1"/>
@@ -3990,30 +3978,30 @@
         <v>46109.449884259258</v>
       </c>
       <c r="S44" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="45" spans="1:19" ht="87.45" customHeight="1">
       <c r="A45" t="s">
-        <v>288</v>
+        <v>251</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>289</v>
+        <v>252</v>
       </c>
       <c r="C45" s="2">
         <v>46109.616851851853</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>290</v>
+        <v>253</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>291</v>
+        <v>380</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>292</v>
+        <v>254</v>
       </c>
       <c r="H45" s="4">
         <v>46079.791666666657</v>
@@ -4025,13 +4013,13 @@
         <v>144000</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>293</v>
+        <v>255</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N45" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="O45" s="6">
         <f t="shared" si="1"/>
@@ -4044,30 +4032,30 @@
         <v>46109.450185185182</v>
       </c>
       <c r="S45" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="46" spans="1:19" ht="102" customHeight="1">
       <c r="A46" t="s">
-        <v>294</v>
+        <v>256</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>295</v>
+        <v>257</v>
       </c>
       <c r="C46" s="2">
         <v>46109.617152777777</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>296</v>
+        <v>258</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>297</v>
+        <v>259</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>298</v>
+        <v>381</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>299</v>
+        <v>260</v>
       </c>
       <c r="H46" s="4">
         <v>46080.791666666657</v>
@@ -4079,13 +4067,13 @@
         <v>174000</v>
       </c>
       <c r="L46" s="1" t="s">
-        <v>300</v>
+        <v>261</v>
       </c>
       <c r="M46" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N46" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O46" s="6">
         <f t="shared" si="1"/>
@@ -4098,30 +4086,30 @@
         <v>46109.450486111113</v>
       </c>
       <c r="S46" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="47" spans="1:19" ht="87.45" customHeight="1">
       <c r="A47" t="s">
-        <v>301</v>
+        <v>262</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>302</v>
+        <v>263</v>
       </c>
       <c r="C47" s="2">
         <v>46109.617430555547</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>303</v>
+        <v>264</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>304</v>
+        <v>382</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>292</v>
+        <v>254</v>
       </c>
       <c r="H47" s="4">
         <v>46079.791666666657</v>
@@ -4133,13 +4121,13 @@
         <v>20000</v>
       </c>
       <c r="L47" s="1" t="s">
-        <v>293</v>
+        <v>255</v>
       </c>
       <c r="M47" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N47" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="O47" s="6">
         <f t="shared" si="1"/>
@@ -4152,30 +4140,30 @@
         <v>46109.45076388889</v>
       </c>
       <c r="S47" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="48" spans="1:19" ht="43.75" customHeight="1">
       <c r="A48" t="s">
-        <v>305</v>
+        <v>265</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>306</v>
+        <v>266</v>
       </c>
       <c r="C48" s="2">
         <v>46109.617650462962</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>307</v>
+        <v>267</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>308</v>
+        <v>383</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>309</v>
+        <v>268</v>
       </c>
       <c r="H48" s="4">
         <v>46079.791666666657</v>
@@ -4187,13 +4175,13 @@
         <v>57000</v>
       </c>
       <c r="L48" s="1" t="s">
-        <v>293</v>
+        <v>255</v>
       </c>
       <c r="M48" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N48" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="O48" s="6">
         <f t="shared" si="1"/>
@@ -4206,30 +4194,30 @@
         <v>46109.450983796298</v>
       </c>
       <c r="S48" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="49" spans="1:19" ht="29.15" customHeight="1">
       <c r="A49" t="s">
-        <v>310</v>
+        <v>269</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>311</v>
+        <v>270</v>
       </c>
       <c r="C49" s="2">
         <v>46109.618298611109</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>312</v>
+        <v>271</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>313</v>
+        <v>272</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>314</v>
+        <v>384</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>315</v>
+        <v>273</v>
       </c>
       <c r="H49" s="4">
         <v>46093.833333333343</v>
@@ -4241,13 +4229,13 @@
         <v>46300</v>
       </c>
       <c r="L49" s="1" t="s">
-        <v>316</v>
+        <v>274</v>
       </c>
       <c r="M49" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N49" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O49" s="6">
         <f t="shared" si="1"/>
@@ -4260,30 +4248,30 @@
         <v>46109.451631944437</v>
       </c>
       <c r="S49" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="50" spans="1:19" ht="43.75" customHeight="1">
       <c r="A50" t="s">
-        <v>317</v>
+        <v>275</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>318</v>
+        <v>276</v>
       </c>
       <c r="C50" s="2">
         <v>46092.908356481479</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>319</v>
+        <v>277</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>161</v>
+        <v>143</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>320</v>
+        <v>385</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>321</v>
+        <v>278</v>
       </c>
       <c r="H50" s="4">
         <v>46271.833333333343</v>
@@ -4295,13 +4283,13 @@
         <v>0</v>
       </c>
       <c r="L50" s="1" t="s">
-        <v>195</v>
+        <v>171</v>
       </c>
       <c r="M50" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N50" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O50" s="6">
         <f t="shared" si="1"/>
@@ -4314,30 +4302,30 @@
         <v>46092.741689814808</v>
       </c>
       <c r="S50" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="51" spans="1:19" ht="29.15" customHeight="1">
       <c r="A51" t="s">
-        <v>322</v>
+        <v>279</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>323</v>
+        <v>280</v>
       </c>
       <c r="C51" s="2">
         <v>46108.883298611108</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>324</v>
+        <v>281</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>325</v>
+        <v>282</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>326</v>
+        <v>386</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>327</v>
+        <v>283</v>
       </c>
       <c r="H51" s="4">
         <v>46121.833333333343</v>
@@ -4349,10 +4337,10 @@
         <v>373000</v>
       </c>
       <c r="M51" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N51" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O51" s="6">
         <f t="shared" si="1"/>
@@ -4365,30 +4353,30 @@
         <v>46108.716631944437</v>
       </c>
       <c r="S51" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="52" spans="1:19" ht="43.75" customHeight="1">
       <c r="A52" t="s">
-        <v>328</v>
+        <v>284</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>329</v>
+        <v>285</v>
       </c>
       <c r="C52" s="2">
         <v>46109.623437499999</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>330</v>
+        <v>286</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>331</v>
+        <v>387</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>332</v>
+        <v>287</v>
       </c>
       <c r="H52" s="4">
         <v>46072.791666666657</v>
@@ -4400,13 +4388,13 @@
         <v>407000</v>
       </c>
       <c r="L52" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M52" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N52" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O52" s="6">
         <f t="shared" si="1"/>
@@ -4419,30 +4407,30 @@
         <v>46109.456770833327</v>
       </c>
       <c r="S52" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="53" spans="1:19" ht="160.30000000000001" customHeight="1">
       <c r="A53" t="s">
-        <v>333</v>
+        <v>288</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>334</v>
+        <v>289</v>
       </c>
       <c r="C53" s="2">
         <v>46109.620324074072</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>335</v>
+        <v>290</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>336</v>
+        <v>291</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>337</v>
+        <v>388</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>338</v>
+        <v>292</v>
       </c>
       <c r="H53" s="4">
         <v>46149.833333333343</v>
@@ -4454,13 +4442,13 @@
         <v>45200</v>
       </c>
       <c r="L53" s="1" t="s">
-        <v>339</v>
+        <v>293</v>
       </c>
       <c r="M53" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N53" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O53" s="6">
         <f t="shared" si="1"/>
@@ -4473,30 +4461,30 @@
         <v>46109.453657407408</v>
       </c>
       <c r="S53" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="54" spans="1:19" ht="43.75" customHeight="1">
       <c r="A54" t="s">
-        <v>340</v>
+        <v>294</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>341</v>
+        <v>295</v>
       </c>
       <c r="C54" s="2">
         <v>46109.620671296303</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>342</v>
+        <v>296</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>343</v>
+        <v>389</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>344</v>
+        <v>297</v>
       </c>
       <c r="H54" s="4">
         <v>46208.833333333343</v>
@@ -4508,13 +4496,13 @@
         <v>222000</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N54" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="O54" s="6">
         <f t="shared" si="1"/>
@@ -4527,27 +4515,30 @@
         <v>46109.454004629632</v>
       </c>
       <c r="S54" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="55" spans="1:19">
       <c r="A55" t="s">
-        <v>345</v>
+        <v>298</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>346</v>
+        <v>299</v>
       </c>
       <c r="C55" s="2">
         <v>46109.630381944437</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>347</v>
+        <v>300</v>
       </c>
       <c r="E55" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="F55" s="3" t="s">
         <v>348</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>349</v>
+        <v>302</v>
       </c>
       <c r="H55" s="4">
         <v>46121.833333333343</v>
@@ -4559,10 +4550,10 @@
         <v>401000</v>
       </c>
       <c r="M55" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N55" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O55" s="6">
         <f t="shared" si="1"/>
@@ -4575,27 +4566,30 @@
         <v>46109.46371527778</v>
       </c>
       <c r="S55" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="56" spans="1:19">
       <c r="A56" t="s">
-        <v>350</v>
+        <v>303</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>351</v>
+        <v>304</v>
       </c>
       <c r="C56" s="2">
         <v>46109.612812500003</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>352</v>
+        <v>305</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>353</v>
+        <v>306</v>
+      </c>
+      <c r="F56" s="3" t="s">
+        <v>348</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>354</v>
+        <v>307</v>
       </c>
       <c r="H56" s="4">
         <v>46051.791666666657</v>
@@ -4607,13 +4601,13 @@
         <v>0</v>
       </c>
       <c r="L56" s="1" t="s">
-        <v>355</v>
+        <v>308</v>
       </c>
       <c r="M56" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N56" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O56" s="6">
         <f t="shared" si="1"/>
@@ -4626,30 +4620,30 @@
         <v>46109.446145833332</v>
       </c>
       <c r="S56" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="57" spans="1:19">
       <c r="A57" t="s">
-        <v>356</v>
+        <v>309</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>357</v>
+        <v>310</v>
       </c>
       <c r="C57" s="2">
         <v>46109.613194444442</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>358</v>
+        <v>311</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>359</v>
+        <v>390</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>360</v>
+        <v>312</v>
       </c>
       <c r="H57" s="4">
         <v>46107.833333333343</v>
@@ -4661,13 +4655,13 @@
         <v>288000</v>
       </c>
       <c r="L57" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M57" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N57" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="O57" s="6">
         <f t="shared" si="1"/>
@@ -4680,30 +4674,30 @@
         <v>46109.446527777778</v>
       </c>
       <c r="S57" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="58" spans="1:19" ht="87.45" customHeight="1">
       <c r="A58" t="s">
-        <v>361</v>
+        <v>313</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>362</v>
+        <v>314</v>
       </c>
       <c r="C58" s="2">
         <v>46092.938900462963</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>363</v>
+        <v>315</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>364</v>
+        <v>391</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>365</v>
+        <v>316</v>
       </c>
       <c r="H58" s="4">
         <v>46100.833333333343</v>
@@ -4715,13 +4709,13 @@
         <v>85200</v>
       </c>
       <c r="L58" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="M58" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N58" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="O58" s="6">
         <f t="shared" si="1"/>
@@ -4734,30 +4728,30 @@
         <v>46092.772233796299</v>
       </c>
       <c r="S58" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="59" spans="1:19" ht="189.45" customHeight="1">
       <c r="A59" t="s">
-        <v>366</v>
+        <v>317</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>367</v>
+        <v>318</v>
       </c>
       <c r="C59" s="2">
         <v>46109.615416666667</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>368</v>
+        <v>319</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>369</v>
+        <v>320</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>370</v>
+        <v>392</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>371</v>
+        <v>321</v>
       </c>
       <c r="H59" s="4">
         <v>46100.833333333343</v>
@@ -4769,13 +4763,13 @@
         <v>53900</v>
       </c>
       <c r="L59" s="1" t="s">
-        <v>372</v>
+        <v>322</v>
       </c>
       <c r="M59" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N59" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O59" s="6">
         <f t="shared" si="1"/>
@@ -4788,30 +4782,30 @@
         <v>46109.448750000003</v>
       </c>
       <c r="S59" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="60" spans="1:19" ht="306" customHeight="1">
       <c r="A60" t="s">
-        <v>373</v>
+        <v>323</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>374</v>
+        <v>324</v>
       </c>
       <c r="C60" s="2">
         <v>46092.557858796303</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>375</v>
+        <v>325</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>376</v>
+        <v>393</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>377</v>
+        <v>326</v>
       </c>
       <c r="H60" s="4">
         <v>46425.791666666657</v>
@@ -4823,13 +4817,13 @@
         <v>65400</v>
       </c>
       <c r="L60" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M60" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N60" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O60" s="6">
         <f t="shared" si="1"/>
@@ -4842,27 +4836,30 @@
         <v>46092.391192129631</v>
       </c>
       <c r="S60" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="61" spans="1:19">
       <c r="A61" t="s">
-        <v>378</v>
+        <v>327</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>379</v>
+        <v>328</v>
       </c>
       <c r="C61" s="2">
         <v>46109.611284722218</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>380</v>
+        <v>329</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>381</v>
+        <v>330</v>
+      </c>
+      <c r="F61" s="3" t="s">
+        <v>348</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>382</v>
+        <v>331</v>
       </c>
       <c r="H61" s="4">
         <v>46100.833333333343</v>
@@ -4874,10 +4871,10 @@
         <v>184000</v>
       </c>
       <c r="M61" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N61" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O61" s="6">
         <f t="shared" si="1"/>
@@ -4890,7 +4887,7 @@
         <v>46109.444618055553</v>
       </c>
       <c r="S61" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -4946,66 +4943,66 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>383</v>
+        <v>332</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>384</v>
+        <v>333</v>
       </c>
       <c r="B2" t="s">
-        <v>385</v>
+        <v>334</v>
       </c>
       <c r="C2" t="s">
-        <v>386</v>
+        <v>335</v>
       </c>
       <c r="D2" t="s">
-        <v>387</v>
+        <v>336</v>
       </c>
       <c r="E2" t="s">
-        <v>388</v>
+        <v>337</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>389</v>
+        <v>338</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>390</v>
+        <v>339</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B4" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C4" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B5" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="C5" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>